<commit_message>
Ajustes para a geração do arquivo de histórico. Todas as bases atualizadas
</commit_message>
<xml_diff>
--- a/Bases/Lista de ações.xlsx
+++ b/Bases/Lista de ações.xlsx
@@ -319,15 +319,15 @@
     <t>Sanepar</t>
   </si>
   <si>
+    <t>Banco Santander</t>
+  </si>
+  <si>
+    <t>Randon</t>
+  </si>
+  <si>
     <t>Recrusul</t>
   </si>
   <si>
-    <t>Banco Santander</t>
-  </si>
-  <si>
-    <t>Randon</t>
-  </si>
-  <si>
     <t>Fleury</t>
   </si>
   <si>
@@ -1288,13 +1288,13 @@
     <t>SAPR4</t>
   </si>
   <si>
+    <t>SANB11</t>
+  </si>
+  <si>
+    <t>RAPT4</t>
+  </si>
+  <si>
     <t>RCSL4</t>
-  </si>
-  <si>
-    <t>SANB11</t>
-  </si>
-  <si>
-    <t>RAPT4</t>
   </si>
   <si>
     <t>FLRY3</t>
@@ -2575,7 +2575,7 @@
         <v>282174900</v>
       </c>
       <c r="D2" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="3" spans="1:4">
@@ -2589,7 +2589,7 @@
         <v>65204900</v>
       </c>
       <c r="D3" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -2603,7 +2603,7 @@
         <v>64731600</v>
       </c>
       <c r="D4" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="5" spans="1:4">
@@ -2617,7 +2617,7 @@
         <v>37935400</v>
       </c>
       <c r="D5" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="6" spans="1:4">
@@ -2631,7 +2631,7 @@
         <v>37609700</v>
       </c>
       <c r="D6" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="7" spans="1:4">
@@ -2642,10 +2642,10 @@
         <v>329</v>
       </c>
       <c r="C7">
-        <v>35795000</v>
+        <v>35795300</v>
       </c>
       <c r="D7" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="8" spans="1:4">
@@ -2659,7 +2659,7 @@
         <v>35579100</v>
       </c>
       <c r="D8" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="9" spans="1:4">
@@ -2673,7 +2673,7 @@
         <v>31760000</v>
       </c>
       <c r="D9" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="10" spans="1:4">
@@ -2687,7 +2687,7 @@
         <v>29781400</v>
       </c>
       <c r="D10" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="11" spans="1:4">
@@ -2701,7 +2701,7 @@
         <v>26227400</v>
       </c>
       <c r="D11" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="12" spans="1:4">
@@ -2715,7 +2715,7 @@
         <v>26162200</v>
       </c>
       <c r="D12" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="13" spans="1:4">
@@ -2726,10 +2726,10 @@
         <v>335</v>
       </c>
       <c r="C13">
-        <v>24978800</v>
+        <v>24980100</v>
       </c>
       <c r="D13" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="14" spans="1:4">
@@ -2743,7 +2743,7 @@
         <v>24151500</v>
       </c>
       <c r="D14" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="15" spans="1:4">
@@ -2757,7 +2757,7 @@
         <v>19383700</v>
       </c>
       <c r="D15" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="16" spans="1:4">
@@ -2768,10 +2768,10 @@
         <v>338</v>
       </c>
       <c r="C16">
-        <v>19134800</v>
+        <v>19129400</v>
       </c>
       <c r="D16" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="17" spans="1:4">
@@ -2785,7 +2785,7 @@
         <v>17884400</v>
       </c>
       <c r="D17" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="18" spans="1:4">
@@ -2799,7 +2799,7 @@
         <v>17748600</v>
       </c>
       <c r="D18" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="19" spans="1:4">
@@ -2813,7 +2813,7 @@
         <v>16986500</v>
       </c>
       <c r="D19" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="20" spans="1:4">
@@ -2827,7 +2827,7 @@
         <v>15879100</v>
       </c>
       <c r="D20" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="21" spans="1:4">
@@ -2841,7 +2841,7 @@
         <v>15628900</v>
       </c>
       <c r="D21" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="22" spans="1:4">
@@ -2855,7 +2855,7 @@
         <v>14692000</v>
       </c>
       <c r="D22" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="23" spans="1:4">
@@ -2869,7 +2869,7 @@
         <v>13749000</v>
       </c>
       <c r="D23" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="24" spans="1:4">
@@ -2883,7 +2883,7 @@
         <v>13331400</v>
       </c>
       <c r="D24" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="25" spans="1:4">
@@ -2897,7 +2897,7 @@
         <v>12487200</v>
       </c>
       <c r="D25" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="26" spans="1:4">
@@ -2911,7 +2911,7 @@
         <v>12271300</v>
       </c>
       <c r="D26" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="27" spans="1:4">
@@ -2925,7 +2925,7 @@
         <v>12026500</v>
       </c>
       <c r="D27" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="28" spans="1:4">
@@ -2939,7 +2939,7 @@
         <v>11836900</v>
       </c>
       <c r="D28" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="29" spans="1:4">
@@ -2953,7 +2953,7 @@
         <v>11655000</v>
       </c>
       <c r="D29" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="30" spans="1:4">
@@ -2967,7 +2967,7 @@
         <v>11649400</v>
       </c>
       <c r="D30" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="31" spans="1:4">
@@ -2981,7 +2981,7 @@
         <v>11489500</v>
       </c>
       <c r="D31" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="32" spans="1:4">
@@ -2995,7 +2995,7 @@
         <v>11241600</v>
       </c>
       <c r="D32" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="33" spans="1:4">
@@ -3009,7 +3009,7 @@
         <v>10892500</v>
       </c>
       <c r="D33" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="34" spans="1:4">
@@ -3020,10 +3020,10 @@
         <v>356</v>
       </c>
       <c r="C34">
-        <v>10867400</v>
+        <v>10867300</v>
       </c>
       <c r="D34" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="35" spans="1:4">
@@ -3037,7 +3037,7 @@
         <v>10623500</v>
       </c>
       <c r="D35" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="36" spans="1:4">
@@ -3051,7 +3051,7 @@
         <v>10483000</v>
       </c>
       <c r="D36" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="37" spans="1:4">
@@ -3065,7 +3065,7 @@
         <v>10397200</v>
       </c>
       <c r="D37" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="38" spans="1:4">
@@ -3079,7 +3079,7 @@
         <v>10363400</v>
       </c>
       <c r="D38" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="39" spans="1:4">
@@ -3090,10 +3090,10 @@
         <v>361</v>
       </c>
       <c r="C39">
-        <v>10241400</v>
+        <v>10241800</v>
       </c>
       <c r="D39" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="40" spans="1:4">
@@ -3107,7 +3107,7 @@
         <v>10032300</v>
       </c>
       <c r="D40" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="41" spans="1:4">
@@ -3121,7 +3121,7 @@
         <v>9985000</v>
       </c>
       <c r="D41" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="42" spans="1:4">
@@ -3132,10 +3132,10 @@
         <v>364</v>
       </c>
       <c r="C42">
-        <v>9898800</v>
+        <v>9900100</v>
       </c>
       <c r="D42" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="43" spans="1:4">
@@ -3149,7 +3149,7 @@
         <v>9629400</v>
       </c>
       <c r="D43" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="44" spans="1:4">
@@ -3160,10 +3160,10 @@
         <v>366</v>
       </c>
       <c r="C44">
-        <v>9537800</v>
+        <v>9538800</v>
       </c>
       <c r="D44" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="45" spans="1:4">
@@ -3177,7 +3177,7 @@
         <v>9144900</v>
       </c>
       <c r="D45" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="46" spans="1:4">
@@ -3188,10 +3188,10 @@
         <v>368</v>
       </c>
       <c r="C46">
-        <v>9077700</v>
+        <v>9070500</v>
       </c>
       <c r="D46" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="47" spans="1:4">
@@ -3205,7 +3205,7 @@
         <v>8816200</v>
       </c>
       <c r="D47" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="48" spans="1:4">
@@ -3219,7 +3219,7 @@
         <v>8768100</v>
       </c>
       <c r="D48" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="49" spans="1:4">
@@ -3230,10 +3230,10 @@
         <v>371</v>
       </c>
       <c r="C49">
-        <v>8555400</v>
+        <v>8556400</v>
       </c>
       <c r="D49" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="50" spans="1:4">
@@ -3247,7 +3247,7 @@
         <v>8418600</v>
       </c>
       <c r="D50" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="51" spans="1:4">
@@ -3261,7 +3261,7 @@
         <v>8327900</v>
       </c>
       <c r="D51" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="52" spans="1:4">
@@ -3275,7 +3275,7 @@
         <v>8269500</v>
       </c>
       <c r="D52" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="53" spans="1:4">
@@ -3289,7 +3289,7 @@
         <v>7971200</v>
       </c>
       <c r="D53" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="54" spans="1:4">
@@ -3303,7 +3303,7 @@
         <v>7962500</v>
       </c>
       <c r="D54" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="55" spans="1:4">
@@ -3317,7 +3317,7 @@
         <v>7926500</v>
       </c>
       <c r="D55" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="56" spans="1:4">
@@ -3331,7 +3331,7 @@
         <v>7878300</v>
       </c>
       <c r="D56" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="57" spans="1:4">
@@ -3342,10 +3342,10 @@
         <v>379</v>
       </c>
       <c r="C57">
-        <v>7618000</v>
+        <v>7620300</v>
       </c>
       <c r="D57" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="58" spans="1:4">
@@ -3359,7 +3359,7 @@
         <v>7437100</v>
       </c>
       <c r="D58" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="59" spans="1:4">
@@ -3370,10 +3370,10 @@
         <v>381</v>
       </c>
       <c r="C59">
-        <v>7158000</v>
+        <v>7129200</v>
       </c>
       <c r="D59" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="60" spans="1:4">
@@ -3387,7 +3387,7 @@
         <v>7115300</v>
       </c>
       <c r="D60" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="61" spans="1:4">
@@ -3401,7 +3401,7 @@
         <v>6961800</v>
       </c>
       <c r="D61" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="62" spans="1:4">
@@ -3415,7 +3415,7 @@
         <v>6715200</v>
       </c>
       <c r="D62" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="63" spans="1:4">
@@ -3429,7 +3429,7 @@
         <v>6563400</v>
       </c>
       <c r="D63" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="64" spans="1:4">
@@ -3443,7 +3443,7 @@
         <v>6212800</v>
       </c>
       <c r="D64" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="65" spans="1:4">
@@ -3457,7 +3457,7 @@
         <v>6092500</v>
       </c>
       <c r="D65" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="66" spans="1:4">
@@ -3471,7 +3471,7 @@
         <v>6043800</v>
       </c>
       <c r="D66" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="67" spans="1:4">
@@ -3485,7 +3485,7 @@
         <v>5957500</v>
       </c>
       <c r="D67" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="68" spans="1:4">
@@ -3499,7 +3499,7 @@
         <v>5928000</v>
       </c>
       <c r="D68" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="69" spans="1:4">
@@ -3513,7 +3513,7 @@
         <v>5707400</v>
       </c>
       <c r="D69" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="70" spans="1:4">
@@ -3527,7 +3527,7 @@
         <v>5601000</v>
       </c>
       <c r="D70" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="71" spans="1:4">
@@ -3538,10 +3538,10 @@
         <v>393</v>
       </c>
       <c r="C71">
-        <v>5484100</v>
+        <v>5485300</v>
       </c>
       <c r="D71" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="72" spans="1:4">
@@ -3555,7 +3555,7 @@
         <v>5424000</v>
       </c>
       <c r="D72" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="73" spans="1:4">
@@ -3569,7 +3569,7 @@
         <v>5128600</v>
       </c>
       <c r="D73" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="74" spans="1:4">
@@ -3583,7 +3583,7 @@
         <v>4929000</v>
       </c>
       <c r="D74" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="75" spans="1:4">
@@ -3597,7 +3597,7 @@
         <v>4899000</v>
       </c>
       <c r="D75" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="76" spans="1:4">
@@ -3608,10 +3608,10 @@
         <v>398</v>
       </c>
       <c r="C76">
-        <v>4671300</v>
+        <v>4671200</v>
       </c>
       <c r="D76" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="77" spans="1:4">
@@ -3625,7 +3625,7 @@
         <v>4611500</v>
       </c>
       <c r="D77" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="78" spans="1:4">
@@ -3639,7 +3639,7 @@
         <v>4551600</v>
       </c>
       <c r="D78" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="79" spans="1:4">
@@ -3653,7 +3653,7 @@
         <v>4547900</v>
       </c>
       <c r="D79" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="80" spans="1:4">
@@ -3667,7 +3667,7 @@
         <v>4513400</v>
       </c>
       <c r="D80" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="81" spans="1:4">
@@ -3681,7 +3681,7 @@
         <v>4379000</v>
       </c>
       <c r="D81" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="82" spans="1:4">
@@ -3692,10 +3692,10 @@
         <v>404</v>
       </c>
       <c r="C82">
-        <v>4202700</v>
+        <v>4202800</v>
       </c>
       <c r="D82" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="83" spans="1:4">
@@ -3709,7 +3709,7 @@
         <v>4195500</v>
       </c>
       <c r="D83" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="84" spans="1:4">
@@ -3723,7 +3723,7 @@
         <v>4070400</v>
       </c>
       <c r="D84" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="85" spans="1:4">
@@ -3737,7 +3737,7 @@
         <v>3959800</v>
       </c>
       <c r="D85" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="86" spans="1:4">
@@ -3751,7 +3751,7 @@
         <v>3739800</v>
       </c>
       <c r="D86" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="87" spans="1:4">
@@ -3765,7 +3765,7 @@
         <v>3705800</v>
       </c>
       <c r="D87" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="88" spans="1:4">
@@ -3779,7 +3779,7 @@
         <v>3641600</v>
       </c>
       <c r="D88" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="89" spans="1:4">
@@ -3793,7 +3793,7 @@
         <v>3588800</v>
       </c>
       <c r="D89" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="90" spans="1:4">
@@ -3807,7 +3807,7 @@
         <v>2971200</v>
       </c>
       <c r="D90" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="91" spans="1:4">
@@ -3821,7 +3821,7 @@
         <v>2840700</v>
       </c>
       <c r="D91" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="92" spans="1:4">
@@ -3835,7 +3835,7 @@
         <v>2827600</v>
       </c>
       <c r="D92" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="93" spans="1:4">
@@ -3849,7 +3849,7 @@
         <v>2826600</v>
       </c>
       <c r="D93" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="94" spans="1:4">
@@ -3863,7 +3863,7 @@
         <v>2763900</v>
       </c>
       <c r="D94" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="95" spans="1:4">
@@ -3877,7 +3877,7 @@
         <v>2718300</v>
       </c>
       <c r="D95" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="96" spans="1:4">
@@ -3888,10 +3888,10 @@
         <v>418</v>
       </c>
       <c r="C96">
-        <v>2652600</v>
+        <v>2652700</v>
       </c>
       <c r="D96" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="97" spans="1:4">
@@ -3905,7 +3905,7 @@
         <v>2650700</v>
       </c>
       <c r="D97" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="98" spans="1:4">
@@ -3919,7 +3919,7 @@
         <v>2614400</v>
       </c>
       <c r="D98" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="99" spans="1:4">
@@ -3933,7 +3933,7 @@
         <v>2449700</v>
       </c>
       <c r="D99" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="100" spans="1:4">
@@ -3947,7 +3947,7 @@
         <v>2445600</v>
       </c>
       <c r="D100" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="101" spans="1:4">
@@ -3961,7 +3961,7 @@
         <v>2411100</v>
       </c>
       <c r="D101" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="102" spans="1:4">
@@ -3972,10 +3972,10 @@
         <v>424</v>
       </c>
       <c r="C102">
-        <v>2328400</v>
+        <v>2324000</v>
       </c>
       <c r="D102" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="103" spans="1:4">
@@ -3986,10 +3986,10 @@
         <v>425</v>
       </c>
       <c r="C103">
-        <v>2324000</v>
+        <v>2302500</v>
       </c>
       <c r="D103" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="104" spans="1:4">
@@ -4000,10 +4000,10 @@
         <v>426</v>
       </c>
       <c r="C104">
-        <v>2302500</v>
+        <v>2298100</v>
       </c>
       <c r="D104" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="105" spans="1:4">
@@ -4017,7 +4017,7 @@
         <v>2274200</v>
       </c>
       <c r="D105" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="106" spans="1:4">
@@ -4031,7 +4031,7 @@
         <v>2271800</v>
       </c>
       <c r="D106" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="107" spans="1:4">
@@ -4045,7 +4045,7 @@
         <v>2127600</v>
       </c>
       <c r="D107" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="108" spans="1:4">
@@ -4059,7 +4059,7 @@
         <v>2098300</v>
       </c>
       <c r="D108" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="109" spans="1:4">
@@ -4073,7 +4073,7 @@
         <v>2083300</v>
       </c>
       <c r="D109" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="110" spans="1:4">
@@ -4087,7 +4087,7 @@
         <v>1993800</v>
       </c>
       <c r="D110" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="111" spans="1:4">
@@ -4101,7 +4101,7 @@
         <v>1977400</v>
       </c>
       <c r="D111" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="112" spans="1:4">
@@ -4112,10 +4112,10 @@
         <v>434</v>
       </c>
       <c r="C112">
-        <v>1954100</v>
+        <v>1952200</v>
       </c>
       <c r="D112" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="113" spans="1:4">
@@ -4126,10 +4126,10 @@
         <v>435</v>
       </c>
       <c r="C113">
-        <v>1939300</v>
+        <v>1939600</v>
       </c>
       <c r="D113" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="114" spans="1:4">
@@ -4143,7 +4143,7 @@
         <v>1920800</v>
       </c>
       <c r="D114" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="115" spans="1:4">
@@ -4157,7 +4157,7 @@
         <v>1885400</v>
       </c>
       <c r="D115" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="116" spans="1:4">
@@ -4171,7 +4171,7 @@
         <v>1844800</v>
       </c>
       <c r="D116" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="117" spans="1:4">
@@ -4185,7 +4185,7 @@
         <v>1835800</v>
       </c>
       <c r="D117" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="118" spans="1:4">
@@ -4199,7 +4199,7 @@
         <v>1817500</v>
       </c>
       <c r="D118" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="119" spans="1:4">
@@ -4213,7 +4213,7 @@
         <v>1810900</v>
       </c>
       <c r="D119" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="120" spans="1:4">
@@ -4227,7 +4227,7 @@
         <v>1808000</v>
       </c>
       <c r="D120" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="121" spans="1:4">
@@ -4241,7 +4241,7 @@
         <v>1795400</v>
       </c>
       <c r="D121" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="122" spans="1:4">
@@ -4255,7 +4255,7 @@
         <v>1724300</v>
       </c>
       <c r="D122" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="123" spans="1:4">
@@ -4269,7 +4269,7 @@
         <v>1676200</v>
       </c>
       <c r="D123" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="124" spans="1:4">
@@ -4283,7 +4283,7 @@
         <v>1602700</v>
       </c>
       <c r="D124" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="125" spans="1:4">
@@ -4297,7 +4297,7 @@
         <v>1587900</v>
       </c>
       <c r="D125" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="126" spans="1:4">
@@ -4311,7 +4311,7 @@
         <v>1587600</v>
       </c>
       <c r="D126" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="127" spans="1:4">
@@ -4325,7 +4325,7 @@
         <v>1584800</v>
       </c>
       <c r="D127" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="128" spans="1:4">
@@ -4339,7 +4339,7 @@
         <v>1455600</v>
       </c>
       <c r="D128" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="129" spans="1:4">
@@ -4353,7 +4353,7 @@
         <v>1433300</v>
       </c>
       <c r="D129" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="130" spans="1:4">
@@ -4367,7 +4367,7 @@
         <v>1414800</v>
       </c>
       <c r="D130" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="131" spans="1:4">
@@ -4381,7 +4381,7 @@
         <v>1243000</v>
       </c>
       <c r="D131" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="132" spans="1:4">
@@ -4395,7 +4395,7 @@
         <v>1235700</v>
       </c>
       <c r="D132" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="133" spans="1:4">
@@ -4409,7 +4409,7 @@
         <v>1235000</v>
       </c>
       <c r="D133" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="134" spans="1:4">
@@ -4423,7 +4423,7 @@
         <v>1175600</v>
       </c>
       <c r="D134" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="135" spans="1:4">
@@ -4437,7 +4437,7 @@
         <v>1156800</v>
       </c>
       <c r="D135" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="136" spans="1:4">
@@ -4451,7 +4451,7 @@
         <v>1146000</v>
       </c>
       <c r="D136" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="137" spans="1:4">
@@ -4462,10 +4462,10 @@
         <v>459</v>
       </c>
       <c r="C137">
-        <v>1139200</v>
+        <v>1139300</v>
       </c>
       <c r="D137" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="138" spans="1:4">
@@ -4479,7 +4479,7 @@
         <v>1123700</v>
       </c>
       <c r="D138" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="139" spans="1:4">
@@ -4493,7 +4493,7 @@
         <v>1116100</v>
       </c>
       <c r="D139" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="140" spans="1:4">
@@ -4507,7 +4507,7 @@
         <v>1064800</v>
       </c>
       <c r="D140" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="141" spans="1:4">
@@ -4521,7 +4521,7 @@
         <v>991800</v>
       </c>
       <c r="D141" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="142" spans="1:4">
@@ -4535,7 +4535,7 @@
         <v>988100</v>
       </c>
       <c r="D142" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="143" spans="1:4">
@@ -4549,7 +4549,7 @@
         <v>975300</v>
       </c>
       <c r="D143" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="144" spans="1:4">
@@ -4560,10 +4560,10 @@
         <v>466</v>
       </c>
       <c r="C144">
-        <v>973000</v>
+        <v>974400</v>
       </c>
       <c r="D144" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="145" spans="1:4">
@@ -4577,7 +4577,7 @@
         <v>944700</v>
       </c>
       <c r="D145" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="146" spans="1:4">
@@ -4591,7 +4591,7 @@
         <v>944300</v>
       </c>
       <c r="D146" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="147" spans="1:4">
@@ -4605,7 +4605,7 @@
         <v>894700</v>
       </c>
       <c r="D147" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="148" spans="1:4">
@@ -4619,7 +4619,7 @@
         <v>882000</v>
       </c>
       <c r="D148" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="149" spans="1:4">
@@ -4633,7 +4633,7 @@
         <v>874800</v>
       </c>
       <c r="D149" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="150" spans="1:4">
@@ -4647,7 +4647,7 @@
         <v>853400</v>
       </c>
       <c r="D150" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="151" spans="1:4">
@@ -4661,7 +4661,7 @@
         <v>815900</v>
       </c>
       <c r="D151" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="152" spans="1:4">
@@ -4675,7 +4675,7 @@
         <v>730600</v>
       </c>
       <c r="D152" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="153" spans="1:4">
@@ -4686,10 +4686,10 @@
         <v>475</v>
       </c>
       <c r="C153">
-        <v>726200</v>
+        <v>728300</v>
       </c>
       <c r="D153" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="154" spans="1:4">
@@ -4703,7 +4703,7 @@
         <v>725000</v>
       </c>
       <c r="D154" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="155" spans="1:4">
@@ -4717,7 +4717,7 @@
         <v>683200</v>
       </c>
       <c r="D155" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="156" spans="1:4">
@@ -4731,7 +4731,7 @@
         <v>657200</v>
       </c>
       <c r="D156" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="157" spans="1:4">
@@ -4745,7 +4745,7 @@
         <v>618400</v>
       </c>
       <c r="D157" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="158" spans="1:4">
@@ -4759,7 +4759,7 @@
         <v>602100</v>
       </c>
       <c r="D158" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="159" spans="1:4">
@@ -4773,7 +4773,7 @@
         <v>600200</v>
       </c>
       <c r="D159" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="160" spans="1:4">
@@ -4787,7 +4787,7 @@
         <v>585700</v>
       </c>
       <c r="D160" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="161" spans="1:4">
@@ -4801,7 +4801,7 @@
         <v>553300</v>
       </c>
       <c r="D161" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="162" spans="1:4">
@@ -4812,10 +4812,10 @@
         <v>484</v>
       </c>
       <c r="C162">
-        <v>533300</v>
+        <v>533200</v>
       </c>
       <c r="D162" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="163" spans="1:4">
@@ -4829,7 +4829,7 @@
         <v>512300</v>
       </c>
       <c r="D163" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="164" spans="1:4">
@@ -4843,7 +4843,7 @@
         <v>483800</v>
       </c>
       <c r="D164" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="165" spans="1:4">
@@ -4857,7 +4857,7 @@
         <v>473300</v>
       </c>
       <c r="D165" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="166" spans="1:4">
@@ -4871,7 +4871,7 @@
         <v>472600</v>
       </c>
       <c r="D166" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="167" spans="1:4">
@@ -4885,7 +4885,7 @@
         <v>472500</v>
       </c>
       <c r="D167" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="168" spans="1:4">
@@ -4899,7 +4899,7 @@
         <v>463600</v>
       </c>
       <c r="D168" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="169" spans="1:4">
@@ -4913,7 +4913,7 @@
         <v>456000</v>
       </c>
       <c r="D169" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="170" spans="1:4">
@@ -4927,7 +4927,7 @@
         <v>448200</v>
       </c>
       <c r="D170" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="171" spans="1:4">
@@ -4941,7 +4941,7 @@
         <v>435400</v>
       </c>
       <c r="D171" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="172" spans="1:4">
@@ -4955,7 +4955,7 @@
         <v>429000</v>
       </c>
       <c r="D172" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="173" spans="1:4">
@@ -4969,7 +4969,7 @@
         <v>414100</v>
       </c>
       <c r="D173" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="174" spans="1:4">
@@ -4983,7 +4983,7 @@
         <v>401200</v>
       </c>
       <c r="D174" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="175" spans="1:4">
@@ -4997,7 +4997,7 @@
         <v>399100</v>
       </c>
       <c r="D175" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="176" spans="1:4">
@@ -5011,7 +5011,7 @@
         <v>384400</v>
       </c>
       <c r="D176" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="177" spans="1:4">
@@ -5025,7 +5025,7 @@
         <v>370500</v>
       </c>
       <c r="D177" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="178" spans="1:4">
@@ -5039,7 +5039,7 @@
         <v>369300</v>
       </c>
       <c r="D178" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="179" spans="1:4">
@@ -5053,7 +5053,7 @@
         <v>366000</v>
       </c>
       <c r="D179" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="180" spans="1:4">
@@ -5067,7 +5067,7 @@
         <v>355100</v>
       </c>
       <c r="D180" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="181" spans="1:4">
@@ -5081,7 +5081,7 @@
         <v>349900</v>
       </c>
       <c r="D181" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="182" spans="1:4">
@@ -5095,7 +5095,7 @@
         <v>336200</v>
       </c>
       <c r="D182" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="183" spans="1:4">
@@ -5109,7 +5109,7 @@
         <v>328600</v>
       </c>
       <c r="D183" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="184" spans="1:4">
@@ -5123,7 +5123,7 @@
         <v>327500</v>
       </c>
       <c r="D184" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="185" spans="1:4">
@@ -5137,7 +5137,7 @@
         <v>326400</v>
       </c>
       <c r="D185" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="186" spans="1:4">
@@ -5151,7 +5151,7 @@
         <v>324000</v>
       </c>
       <c r="D186" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="187" spans="1:4">
@@ -5165,7 +5165,7 @@
         <v>322700</v>
       </c>
       <c r="D187" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="188" spans="1:4">
@@ -5179,7 +5179,7 @@
         <v>314500</v>
       </c>
       <c r="D188" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="189" spans="1:4">
@@ -5193,7 +5193,7 @@
         <v>304000</v>
       </c>
       <c r="D189" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="190" spans="1:4">
@@ -5207,12 +5207,12 @@
         <v>299800</v>
       </c>
       <c r="D190" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="191" spans="1:4">
       <c r="A191" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="B191" t="s">
         <v>513</v>
@@ -5221,7 +5221,7 @@
         <v>298700</v>
       </c>
       <c r="D191" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="192" spans="1:4">
@@ -5235,7 +5235,7 @@
         <v>284200</v>
       </c>
       <c r="D192" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="193" spans="1:4">
@@ -5249,7 +5249,7 @@
         <v>274700</v>
       </c>
       <c r="D193" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="194" spans="1:4">
@@ -5263,7 +5263,7 @@
         <v>271200</v>
       </c>
       <c r="D194" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="195" spans="1:4">
@@ -5277,7 +5277,7 @@
         <v>270200</v>
       </c>
       <c r="D195" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="196" spans="1:4">
@@ -5291,7 +5291,7 @@
         <v>252400</v>
       </c>
       <c r="D196" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="197" spans="1:4">
@@ -5305,7 +5305,7 @@
         <v>249300</v>
       </c>
       <c r="D197" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="198" spans="1:4">
@@ -5319,7 +5319,7 @@
         <v>246800</v>
       </c>
       <c r="D198" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="199" spans="1:4">
@@ -5333,7 +5333,7 @@
         <v>236600</v>
       </c>
       <c r="D199" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="200" spans="1:4">
@@ -5344,10 +5344,10 @@
         <v>522</v>
       </c>
       <c r="C200">
-        <v>233900</v>
+        <v>234200</v>
       </c>
       <c r="D200" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="201" spans="1:4">
@@ -5361,7 +5361,7 @@
         <v>232500</v>
       </c>
       <c r="D201" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="202" spans="1:4">
@@ -5375,7 +5375,7 @@
         <v>219200</v>
       </c>
       <c r="D202" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="203" spans="1:4">
@@ -5389,7 +5389,7 @@
         <v>206900</v>
       </c>
       <c r="D203" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="204" spans="1:4">
@@ -5403,7 +5403,7 @@
         <v>206900</v>
       </c>
       <c r="D204" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="205" spans="1:4">
@@ -5417,7 +5417,7 @@
         <v>203900</v>
       </c>
       <c r="D205" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="206" spans="1:4">
@@ -5431,7 +5431,7 @@
         <v>202800</v>
       </c>
       <c r="D206" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="207" spans="1:4">
@@ -5445,7 +5445,7 @@
         <v>202300</v>
       </c>
       <c r="D207" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="208" spans="1:4">
@@ -5459,7 +5459,7 @@
         <v>196400</v>
       </c>
       <c r="D208" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="209" spans="1:4">
@@ -5473,7 +5473,7 @@
         <v>194300</v>
       </c>
       <c r="D209" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="210" spans="1:4">
@@ -5487,7 +5487,7 @@
         <v>191400</v>
       </c>
       <c r="D210" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="211" spans="1:4">
@@ -5501,7 +5501,7 @@
         <v>189700</v>
       </c>
       <c r="D211" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="212" spans="1:4">
@@ -5515,7 +5515,7 @@
         <v>188900</v>
       </c>
       <c r="D212" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="213" spans="1:4">
@@ -5529,7 +5529,7 @@
         <v>187000</v>
       </c>
       <c r="D213" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="214" spans="1:4">
@@ -5543,7 +5543,7 @@
         <v>183900</v>
       </c>
       <c r="D214" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="215" spans="1:4">
@@ -5557,7 +5557,7 @@
         <v>176100</v>
       </c>
       <c r="D215" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="216" spans="1:4">
@@ -5571,7 +5571,7 @@
         <v>164700</v>
       </c>
       <c r="D216" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="217" spans="1:4">
@@ -5585,7 +5585,7 @@
         <v>162800</v>
       </c>
       <c r="D217" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="218" spans="1:4">
@@ -5599,7 +5599,7 @@
         <v>133000</v>
       </c>
       <c r="D218" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="219" spans="1:4">
@@ -5613,7 +5613,7 @@
         <v>125400</v>
       </c>
       <c r="D219" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="220" spans="1:4">
@@ -5627,7 +5627,7 @@
         <v>123800</v>
       </c>
       <c r="D220" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="221" spans="1:4">
@@ -5641,12 +5641,12 @@
         <v>111800</v>
       </c>
       <c r="D221" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="222" spans="1:4">
       <c r="A222" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B222" t="s">
         <v>544</v>
@@ -5655,7 +5655,7 @@
         <v>101200</v>
       </c>
       <c r="D222" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="223" spans="1:4">
@@ -5669,7 +5669,7 @@
         <v>99600</v>
       </c>
       <c r="D223" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="224" spans="1:4">
@@ -5683,7 +5683,7 @@
         <v>98600</v>
       </c>
       <c r="D224" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="225" spans="1:4">
@@ -5697,7 +5697,7 @@
         <v>96200</v>
       </c>
       <c r="D225" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="226" spans="1:4">
@@ -5711,7 +5711,7 @@
         <v>95100</v>
       </c>
       <c r="D226" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="227" spans="1:4">
@@ -5725,7 +5725,7 @@
         <v>93700</v>
       </c>
       <c r="D227" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="228" spans="1:4">
@@ -5739,7 +5739,7 @@
         <v>91800</v>
       </c>
       <c r="D228" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="229" spans="1:4">
@@ -5753,7 +5753,7 @@
         <v>90700</v>
       </c>
       <c r="D229" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="230" spans="1:4">
@@ -5764,10 +5764,10 @@
         <v>552</v>
       </c>
       <c r="C230">
-        <v>83000</v>
+        <v>83500</v>
       </c>
       <c r="D230" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="231" spans="1:4">
@@ -5781,7 +5781,7 @@
         <v>71100</v>
       </c>
       <c r="D231" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="232" spans="1:4">
@@ -5795,7 +5795,7 @@
         <v>69900</v>
       </c>
       <c r="D232" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="233" spans="1:4">
@@ -5809,12 +5809,12 @@
         <v>69300</v>
       </c>
       <c r="D233" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="234" spans="1:4">
       <c r="A234" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B234" t="s">
         <v>556</v>
@@ -5823,7 +5823,7 @@
         <v>68400</v>
       </c>
       <c r="D234" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="235" spans="1:4">
@@ -5837,7 +5837,7 @@
         <v>66600</v>
       </c>
       <c r="D235" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="236" spans="1:4">
@@ -5851,7 +5851,7 @@
         <v>66600</v>
       </c>
       <c r="D236" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="237" spans="1:4">
@@ -5865,7 +5865,7 @@
         <v>63400</v>
       </c>
       <c r="D237" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="238" spans="1:4">
@@ -5879,7 +5879,7 @@
         <v>63200</v>
       </c>
       <c r="D238" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="239" spans="1:4">
@@ -5893,7 +5893,7 @@
         <v>59800</v>
       </c>
       <c r="D239" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="240" spans="1:4">
@@ -5907,7 +5907,7 @@
         <v>54600</v>
       </c>
       <c r="D240" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="241" spans="1:4">
@@ -5921,7 +5921,7 @@
         <v>52800</v>
       </c>
       <c r="D241" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="242" spans="1:4">
@@ -5932,10 +5932,10 @@
         <v>564</v>
       </c>
       <c r="C242">
-        <v>48000</v>
+        <v>48100</v>
       </c>
       <c r="D242" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="243" spans="1:4">
@@ -5949,7 +5949,7 @@
         <v>46200</v>
       </c>
       <c r="D243" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="244" spans="1:4">
@@ -5963,7 +5963,7 @@
         <v>45600</v>
       </c>
       <c r="D244" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="245" spans="1:4">
@@ -5977,7 +5977,7 @@
         <v>45100</v>
       </c>
       <c r="D245" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="246" spans="1:4">
@@ -5991,7 +5991,7 @@
         <v>39000</v>
       </c>
       <c r="D246" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="247" spans="1:4">
@@ -6005,7 +6005,7 @@
         <v>37600</v>
       </c>
       <c r="D247" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="248" spans="1:4">
@@ -6019,7 +6019,7 @@
         <v>36300</v>
       </c>
       <c r="D248" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="249" spans="1:4">
@@ -6033,7 +6033,7 @@
         <v>35600</v>
       </c>
       <c r="D249" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="250" spans="1:4">
@@ -6047,7 +6047,7 @@
         <v>33900</v>
       </c>
       <c r="D250" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="251" spans="1:4">
@@ -6061,7 +6061,7 @@
         <v>32800</v>
       </c>
       <c r="D251" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="252" spans="1:4">
@@ -6075,7 +6075,7 @@
         <v>32800</v>
       </c>
       <c r="D252" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="253" spans="1:4">
@@ -6089,7 +6089,7 @@
         <v>31800</v>
       </c>
       <c r="D253" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="254" spans="1:4">
@@ -6103,7 +6103,7 @@
         <v>27800</v>
       </c>
       <c r="D254" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="255" spans="1:4">
@@ -6117,7 +6117,7 @@
         <v>27500</v>
       </c>
       <c r="D255" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="256" spans="1:4">
@@ -6131,7 +6131,7 @@
         <v>25300</v>
       </c>
       <c r="D256" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="257" spans="1:4">
@@ -6145,7 +6145,7 @@
         <v>23100</v>
       </c>
       <c r="D257" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="258" spans="1:4">
@@ -6159,7 +6159,7 @@
         <v>20200</v>
       </c>
       <c r="D258" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="259" spans="1:4">
@@ -6173,7 +6173,7 @@
         <v>20100</v>
       </c>
       <c r="D259" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="260" spans="1:4">
@@ -6187,7 +6187,7 @@
         <v>19800</v>
       </c>
       <c r="D260" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="261" spans="1:4">
@@ -6201,7 +6201,7 @@
         <v>17300</v>
       </c>
       <c r="D261" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="262" spans="1:4">
@@ -6215,7 +6215,7 @@
         <v>17200</v>
       </c>
       <c r="D262" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="263" spans="1:4">
@@ -6229,7 +6229,7 @@
         <v>17000</v>
       </c>
       <c r="D263" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="264" spans="1:4">
@@ -6243,7 +6243,7 @@
         <v>16900</v>
       </c>
       <c r="D264" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="265" spans="1:4">
@@ -6257,7 +6257,7 @@
         <v>16400</v>
       </c>
       <c r="D265" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="266" spans="1:4">
@@ -6271,7 +6271,7 @@
         <v>15800</v>
       </c>
       <c r="D266" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="267" spans="1:4">
@@ -6285,7 +6285,7 @@
         <v>15000</v>
       </c>
       <c r="D267" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="268" spans="1:4">
@@ -6299,7 +6299,7 @@
         <v>14100</v>
       </c>
       <c r="D268" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="269" spans="1:4">
@@ -6313,7 +6313,7 @@
         <v>13900</v>
       </c>
       <c r="D269" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="270" spans="1:4">
@@ -6327,7 +6327,7 @@
         <v>13400</v>
       </c>
       <c r="D270" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="271" spans="1:4">
@@ -6341,7 +6341,7 @@
         <v>12800</v>
       </c>
       <c r="D271" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="272" spans="1:4">
@@ -6352,10 +6352,10 @@
         <v>594</v>
       </c>
       <c r="C272">
-        <v>12100</v>
+        <v>12200</v>
       </c>
       <c r="D272" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="273" spans="1:4">
@@ -6369,7 +6369,7 @@
         <v>12000</v>
       </c>
       <c r="D273" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="274" spans="1:4">
@@ -6383,7 +6383,7 @@
         <v>11800</v>
       </c>
       <c r="D274" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="275" spans="1:4">
@@ -6397,12 +6397,12 @@
         <v>11700</v>
       </c>
       <c r="D275" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="276" spans="1:4">
       <c r="A276" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B276" t="s">
         <v>598</v>
@@ -6411,7 +6411,7 @@
         <v>11000</v>
       </c>
       <c r="D276" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="277" spans="1:4">
@@ -6425,7 +6425,7 @@
         <v>10800</v>
       </c>
       <c r="D277" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="278" spans="1:4">
@@ -6439,7 +6439,7 @@
         <v>10300</v>
       </c>
       <c r="D278" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="279" spans="1:4">
@@ -6453,7 +6453,7 @@
         <v>10200</v>
       </c>
       <c r="D279" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="280" spans="1:4">
@@ -6467,7 +6467,7 @@
         <v>10000</v>
       </c>
       <c r="D280" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="281" spans="1:4">
@@ -6481,7 +6481,7 @@
         <v>9900</v>
       </c>
       <c r="D281" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="282" spans="1:4">
@@ -6495,7 +6495,7 @@
         <v>9200</v>
       </c>
       <c r="D282" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="283" spans="1:4">
@@ -6509,7 +6509,7 @@
         <v>9200</v>
       </c>
       <c r="D283" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="284" spans="1:4">
@@ -6523,7 +6523,7 @@
         <v>7600</v>
       </c>
       <c r="D284" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="285" spans="1:4">
@@ -6537,7 +6537,7 @@
         <v>7400</v>
       </c>
       <c r="D285" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="286" spans="1:4">
@@ -6551,7 +6551,7 @@
         <v>6600</v>
       </c>
       <c r="D286" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="287" spans="1:4">
@@ -6565,7 +6565,7 @@
         <v>6400</v>
       </c>
       <c r="D287" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="288" spans="1:4">
@@ -6579,7 +6579,7 @@
         <v>6100</v>
       </c>
       <c r="D288" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="289" spans="1:4">
@@ -6593,7 +6593,7 @@
         <v>5200</v>
       </c>
       <c r="D289" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="290" spans="1:4">
@@ -6607,7 +6607,7 @@
         <v>5100</v>
       </c>
       <c r="D290" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="291" spans="1:4">
@@ -6621,7 +6621,7 @@
         <v>4900</v>
       </c>
       <c r="D291" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="292" spans="1:4">
@@ -6635,7 +6635,7 @@
         <v>4800</v>
       </c>
       <c r="D292" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="293" spans="1:4">
@@ -6649,7 +6649,7 @@
         <v>4800</v>
       </c>
       <c r="D293" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="294" spans="1:4">
@@ -6663,7 +6663,7 @@
         <v>4700</v>
       </c>
       <c r="D294" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="295" spans="1:4">
@@ -6677,7 +6677,7 @@
         <v>4400</v>
       </c>
       <c r="D295" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="296" spans="1:4">
@@ -6691,7 +6691,7 @@
         <v>4400</v>
       </c>
       <c r="D296" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="297" spans="1:4">
@@ -6705,7 +6705,7 @@
         <v>4300</v>
       </c>
       <c r="D297" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="298" spans="1:4">
@@ -6719,7 +6719,7 @@
         <v>3800</v>
       </c>
       <c r="D298" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="299" spans="1:4">
@@ -6733,7 +6733,7 @@
         <v>3800</v>
       </c>
       <c r="D299" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="300" spans="1:4">
@@ -6747,7 +6747,7 @@
         <v>3800</v>
       </c>
       <c r="D300" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="301" spans="1:4">
@@ -6761,7 +6761,7 @@
         <v>3500</v>
       </c>
       <c r="D301" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="302" spans="1:4">
@@ -6775,7 +6775,7 @@
         <v>3300</v>
       </c>
       <c r="D302" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="303" spans="1:4">
@@ -6789,7 +6789,7 @@
         <v>2800</v>
       </c>
       <c r="D303" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="304" spans="1:4">
@@ -6803,7 +6803,7 @@
         <v>2700</v>
       </c>
       <c r="D304" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="305" spans="1:4">
@@ -6817,7 +6817,7 @@
         <v>2400</v>
       </c>
       <c r="D305" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="306" spans="1:4">
@@ -6831,7 +6831,7 @@
         <v>2300</v>
       </c>
       <c r="D306" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="307" spans="1:4">
@@ -6845,7 +6845,7 @@
         <v>2000</v>
       </c>
       <c r="D307" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="308" spans="1:4">
@@ -6859,7 +6859,7 @@
         <v>2000</v>
       </c>
       <c r="D308" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="309" spans="1:4">
@@ -6873,7 +6873,7 @@
         <v>1900</v>
       </c>
       <c r="D309" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="310" spans="1:4">
@@ -6887,7 +6887,7 @@
         <v>1900</v>
       </c>
       <c r="D310" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="311" spans="1:4">
@@ -6901,7 +6901,7 @@
         <v>1700</v>
       </c>
       <c r="D311" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="312" spans="1:4">
@@ -6915,7 +6915,7 @@
         <v>1700</v>
       </c>
       <c r="D312" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="313" spans="1:4">
@@ -6929,7 +6929,7 @@
         <v>1700</v>
       </c>
       <c r="D313" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="314" spans="1:4">
@@ -6943,7 +6943,7 @@
         <v>1700</v>
       </c>
       <c r="D314" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="315" spans="1:4">
@@ -6957,7 +6957,7 @@
         <v>1600</v>
       </c>
       <c r="D315" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="316" spans="1:4">
@@ -6971,7 +6971,7 @@
         <v>1600</v>
       </c>
       <c r="D316" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="317" spans="1:4">
@@ -6985,7 +6985,7 @@
         <v>1400</v>
       </c>
       <c r="D317" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="318" spans="1:4">
@@ -6999,7 +6999,7 @@
         <v>1200</v>
       </c>
       <c r="D318" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="319" spans="1:4">
@@ -7013,7 +7013,7 @@
         <v>1200</v>
       </c>
       <c r="D319" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="320" spans="1:4">
@@ -7027,7 +7027,7 @@
         <v>1200</v>
       </c>
       <c r="D320" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="321" spans="1:4">
@@ -7041,7 +7041,7 @@
         <v>1100</v>
       </c>
       <c r="D321" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="322" spans="1:4">
@@ -7055,7 +7055,7 @@
         <v>1100</v>
       </c>
       <c r="D322" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="323" spans="1:4">
@@ -7069,7 +7069,7 @@
         <v>1100</v>
       </c>
       <c r="D323" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="324" spans="1:4">
@@ -7083,7 +7083,7 @@
         <v>900</v>
       </c>
       <c r="D324" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="325" spans="1:4">
@@ -7097,7 +7097,7 @@
         <v>800</v>
       </c>
       <c r="D325" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="326" spans="1:4">
@@ -7111,7 +7111,7 @@
         <v>800</v>
       </c>
       <c r="D326" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="327" spans="1:4">
@@ -7125,7 +7125,7 @@
         <v>700</v>
       </c>
       <c r="D327" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="328" spans="1:4">
@@ -7139,7 +7139,7 @@
         <v>700</v>
       </c>
       <c r="D328" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="329" spans="1:4">
@@ -7153,7 +7153,7 @@
         <v>600</v>
       </c>
       <c r="D329" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="330" spans="1:4">
@@ -7167,7 +7167,7 @@
         <v>600</v>
       </c>
       <c r="D330" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="331" spans="1:4">
@@ -7181,7 +7181,7 @@
         <v>500</v>
       </c>
       <c r="D331" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="332" spans="1:4">
@@ -7195,7 +7195,7 @@
         <v>500</v>
       </c>
       <c r="D332" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="333" spans="1:4">
@@ -7209,7 +7209,7 @@
         <v>500</v>
       </c>
       <c r="D333" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="334" spans="1:4">
@@ -7223,7 +7223,7 @@
         <v>400</v>
       </c>
       <c r="D334" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="335" spans="1:4">
@@ -7237,7 +7237,7 @@
         <v>300</v>
       </c>
       <c r="D335" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="336" spans="1:4">
@@ -7251,7 +7251,7 @@
         <v>300</v>
       </c>
       <c r="D336" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="337" spans="1:4">
@@ -7265,7 +7265,7 @@
         <v>300</v>
       </c>
       <c r="D337" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="338" spans="1:4">
@@ -7279,7 +7279,7 @@
         <v>300</v>
       </c>
       <c r="D338" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="339" spans="1:4">
@@ -7293,7 +7293,7 @@
         <v>200</v>
       </c>
       <c r="D339" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="340" spans="1:4">
@@ -7307,7 +7307,7 @@
         <v>100</v>
       </c>
       <c r="D340" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="341" spans="1:4">
@@ -7321,7 +7321,7 @@
         <v>100</v>
       </c>
       <c r="D341" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="342" spans="1:4">
@@ -7335,7 +7335,7 @@
         <v>100</v>
       </c>
       <c r="D342" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="343" spans="1:4">
@@ -7349,7 +7349,7 @@
         <v>100</v>
       </c>
       <c r="D343" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="344" spans="1:4">
@@ -7363,7 +7363,7 @@
         <v>100</v>
       </c>
       <c r="D344" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="345" spans="1:4">
@@ -7377,7 +7377,7 @@
         <v>100</v>
       </c>
       <c r="D345" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="346" spans="1:4">
@@ -7391,7 +7391,7 @@
         <v>100</v>
       </c>
       <c r="D346" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="347" spans="1:4">
@@ -7405,7 +7405,7 @@
         <v>100</v>
       </c>
       <c r="D347" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="348" spans="1:4">
@@ -7419,7 +7419,7 @@
         <v>100</v>
       </c>
       <c r="D348" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="349" spans="1:4">
@@ -7433,7 +7433,7 @@
         <v>100</v>
       </c>
       <c r="D349" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="350" spans="1:4">
@@ -7447,7 +7447,7 @@
         <v>100</v>
       </c>
       <c r="D350" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="351" spans="1:4">
@@ -7461,7 +7461,7 @@
         <v>100</v>
       </c>
       <c r="D351" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="352" spans="1:4">
@@ -7475,7 +7475,7 @@
         <v>100</v>
       </c>
       <c r="D352" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="353" spans="1:4">
@@ -7489,7 +7489,7 @@
         <v>100</v>
       </c>
       <c r="D353" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="354" spans="1:4">
@@ -7503,7 +7503,7 @@
         <v>100</v>
       </c>
       <c r="D354" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="355" spans="1:4">
@@ -7517,7 +7517,7 @@
         <v>100</v>
       </c>
       <c r="D355" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="356" spans="1:4">
@@ -7531,7 +7531,7 @@
         <v>42</v>
       </c>
       <c r="D356" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="357" spans="1:4">
@@ -7545,7 +7545,7 @@
         <v>36</v>
       </c>
       <c r="D357" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="358" spans="1:4">
@@ -7559,7 +7559,7 @@
         <v>1000</v>
       </c>
       <c r="D358" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="359" spans="1:4">
@@ -7573,7 +7573,7 @@
         <v>800</v>
       </c>
       <c r="D359" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="360" spans="1:4">
@@ -7587,7 +7587,7 @@
         <v>500</v>
       </c>
       <c r="D360" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="361" spans="1:4">
@@ -7601,7 +7601,7 @@
         <v>400</v>
       </c>
       <c r="D361" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="362" spans="1:4">
@@ -7615,7 +7615,7 @@
         <v>300</v>
       </c>
       <c r="D362" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="363" spans="1:4">
@@ -7629,7 +7629,7 @@
         <v>300</v>
       </c>
       <c r="D363" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="364" spans="1:4">
@@ -7643,7 +7643,7 @@
         <v>300</v>
       </c>
       <c r="D364" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="365" spans="1:4">
@@ -7657,7 +7657,7 @@
         <v>200</v>
       </c>
       <c r="D365" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="366" spans="1:4">
@@ -7671,7 +7671,7 @@
         <v>200</v>
       </c>
       <c r="D366" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="367" spans="1:4">
@@ -7685,7 +7685,7 @@
         <v>200</v>
       </c>
       <c r="D367" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="368" spans="1:4">
@@ -7699,7 +7699,7 @@
         <v>200</v>
       </c>
       <c r="D368" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="369" spans="1:4">
@@ -7713,7 +7713,7 @@
         <v>200</v>
       </c>
       <c r="D369" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="370" spans="1:4">
@@ -7727,7 +7727,7 @@
         <v>100</v>
       </c>
       <c r="D370" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="371" spans="1:4">
@@ -7741,7 +7741,7 @@
         <v>100</v>
       </c>
       <c r="D371" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="372" spans="1:4">
@@ -7755,7 +7755,7 @@
         <v>100</v>
       </c>
       <c r="D372" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="373" spans="1:4">
@@ -7769,7 +7769,7 @@
         <v>100</v>
       </c>
       <c r="D373" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="374" spans="1:4">
@@ -7783,7 +7783,7 @@
         <v>100</v>
       </c>
       <c r="D374" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="375" spans="1:4">
@@ -7797,7 +7797,7 @@
         <v>100</v>
       </c>
       <c r="D375" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="376" spans="1:4">
@@ -7811,7 +7811,7 @@
         <v>5900</v>
       </c>
       <c r="D376" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="377" spans="1:4">
@@ -7825,7 +7825,7 @@
         <v>600</v>
       </c>
       <c r="D377" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="378" spans="1:4">
@@ -7839,7 +7839,7 @@
         <v>500</v>
       </c>
       <c r="D378" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="379" spans="1:4">
@@ -7853,7 +7853,7 @@
         <v>400</v>
       </c>
       <c r="D379" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="380" spans="1:4">
@@ -7867,7 +7867,7 @@
         <v>400</v>
       </c>
       <c r="D380" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="381" spans="1:4">
@@ -7881,7 +7881,7 @@
         <v>300</v>
       </c>
       <c r="D381" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="382" spans="1:4">
@@ -7895,7 +7895,7 @@
         <v>100</v>
       </c>
       <c r="D382" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="383" spans="1:4">
@@ -7909,7 +7909,7 @@
         <v>100</v>
       </c>
       <c r="D383" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="384" spans="1:4">
@@ -7923,7 +7923,7 @@
         <v>100</v>
       </c>
       <c r="D384" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="385" spans="1:4">
@@ -7937,7 +7937,7 @@
         <v>100</v>
       </c>
       <c r="D385" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="386" spans="1:4">
@@ -7951,7 +7951,7 @@
         <v>1500</v>
       </c>
       <c r="D386" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="387" spans="1:4">
@@ -7965,7 +7965,7 @@
         <v>800</v>
       </c>
       <c r="D387" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="388" spans="1:4">
@@ -7979,7 +7979,7 @@
         <v>100</v>
       </c>
       <c r="D388" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="389" spans="1:4">
@@ -7993,7 +7993,7 @@
         <v>14200</v>
       </c>
       <c r="D389" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="390" spans="1:4">
@@ -8007,7 +8007,7 @@
         <v>400</v>
       </c>
       <c r="D390" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="391" spans="1:4">
@@ -8021,7 +8021,7 @@
         <v>200</v>
       </c>
       <c r="D391" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="392" spans="1:4">
@@ -8035,7 +8035,7 @@
         <v>200</v>
       </c>
       <c r="D392" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="393" spans="1:4">
@@ -8049,7 +8049,7 @@
         <v>100</v>
       </c>
       <c r="D393" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="394" spans="1:4">
@@ -8063,7 +8063,7 @@
         <v>100</v>
       </c>
       <c r="D394" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="395" spans="1:4">
@@ -8077,7 +8077,7 @@
         <v>100</v>
       </c>
       <c r="D395" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="396" spans="1:4">
@@ -8091,7 +8091,7 @@
         <v>100</v>
       </c>
       <c r="D396" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="397" spans="1:4">
@@ -8105,7 +8105,7 @@
         <v>100</v>
       </c>
       <c r="D397" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="398" spans="1:4">
@@ -8119,7 +8119,7 @@
         <v>100</v>
       </c>
       <c r="D398" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="399" spans="1:4">
@@ -8133,7 +8133,7 @@
         <v>100</v>
       </c>
       <c r="D399" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="400" spans="1:4">
@@ -8147,7 +8147,7 @@
         <v>200</v>
       </c>
       <c r="D400" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="401" spans="1:4">
@@ -8161,7 +8161,7 @@
         <v>100</v>
       </c>
       <c r="D401" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="402" spans="1:4">
@@ -8175,7 +8175,7 @@
         <v>100</v>
       </c>
       <c r="D402" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="403" spans="1:4">
@@ -8189,7 +8189,7 @@
         <v>20000</v>
       </c>
       <c r="D403" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
     <row r="404" spans="1:4">
@@ -8203,7 +8203,7 @@
         <v>100</v>
       </c>
       <c r="D404" s="2">
-        <v>45773</v>
+        <v>45774</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
- README.md atualizado para incluir novas estratégias de análise e tarefas concluídas; - Modificado “Top 5 ações.txt” para alterar a terminologia de “Média” para “Preço médio” e “Valor de fechamento” para “Preço de fechamento” - "detectar_martelos.py" refatorado para agilizar a plotagem de regressão e remover o código de plotagem não utilizado. - Introduzida uma nova função "plotar_grafico_regressao" em "realizar_analises.py" para melhor visualização da regressão.
</commit_message>
<xml_diff>
--- a/Bases/Lista de ações.xlsx
+++ b/Bases/Lista de ações.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="802" uniqueCount="718">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="800" uniqueCount="717">
   <si>
     <t>Nome da Empresa</t>
   </si>
@@ -304,12 +304,12 @@
     <t>GPS</t>
   </si>
   <si>
+    <t>Camil Alimentos</t>
+  </si>
+  <si>
     <t>Casas Bahia</t>
   </si>
   <si>
-    <t>Camil Alimentos</t>
-  </si>
-  <si>
     <t>Recrusul</t>
   </si>
   <si>
@@ -394,15 +394,15 @@
     <t>CPFL Energia</t>
   </si>
   <si>
+    <t>IRB Brasil RE</t>
+  </si>
+  <si>
+    <t>Mitre Realty</t>
+  </si>
+  <si>
     <t>Azevedo &amp; Travassos</t>
   </si>
   <si>
-    <t>IRB Brasil RE</t>
-  </si>
-  <si>
-    <t>Mitre Realty</t>
-  </si>
-  <si>
     <t>Zamp</t>
   </si>
   <si>
@@ -673,6 +673,9 @@
     <t>Terra Santa</t>
   </si>
   <si>
+    <t>Iguatemi</t>
+  </si>
+  <si>
     <t>Dexxos</t>
   </si>
   <si>
@@ -796,12 +799,12 @@
     <t>Nutriplant</t>
   </si>
   <si>
+    <t>REAG3</t>
+  </si>
+  <si>
     <t>Celesc</t>
   </si>
   <si>
-    <t>REAG3</t>
-  </si>
-  <si>
     <t>Cedro Têxtil</t>
   </si>
   <si>
@@ -889,9 +892,6 @@
     <t>Baumer</t>
   </si>
   <si>
-    <t>Iguatemi</t>
-  </si>
-  <si>
     <t>Equatorial Energia Pará</t>
   </si>
   <si>
@@ -1264,12 +1264,12 @@
     <t>GGPS3</t>
   </si>
   <si>
+    <t>CAML3</t>
+  </si>
+  <si>
     <t>BHIA3</t>
   </si>
   <si>
-    <t>CAML3</t>
-  </si>
-  <si>
     <t>RCSL4</t>
   </si>
   <si>
@@ -1360,15 +1360,15 @@
     <t>CPFE3</t>
   </si>
   <si>
+    <t>IRBR3</t>
+  </si>
+  <si>
+    <t>MTRE3</t>
+  </si>
+  <si>
     <t>AZEV3</t>
   </si>
   <si>
-    <t>IRBR3</t>
-  </si>
-  <si>
-    <t>MTRE3</t>
-  </si>
-  <si>
     <t>ZAMP3</t>
   </si>
   <si>
@@ -2165,9 +2165,6 @@
   </si>
   <si>
     <t>CBEE3</t>
-  </si>
-  <si>
-    <t>RPAD3</t>
   </si>
 </sst>
 </file>
@@ -2529,7 +2526,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D400"/>
+  <dimension ref="A1:D399"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:4">
@@ -2554,10 +2551,10 @@
         <v>321</v>
       </c>
       <c r="C2">
-        <v>121193800</v>
+        <v>121193500</v>
       </c>
       <c r="D2" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="3" spans="1:4">
@@ -2571,7 +2568,7 @@
         <v>117295800</v>
       </c>
       <c r="D3" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -2582,10 +2579,10 @@
         <v>323</v>
       </c>
       <c r="C4">
-        <v>110985700</v>
+        <v>110968400</v>
       </c>
       <c r="D4" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="5" spans="1:4">
@@ -2599,7 +2596,7 @@
         <v>87134400</v>
       </c>
       <c r="D5" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="6" spans="1:4">
@@ -2613,7 +2610,7 @@
         <v>69490700</v>
       </c>
       <c r="D6" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="7" spans="1:4">
@@ -2624,10 +2621,10 @@
         <v>326</v>
       </c>
       <c r="C7">
-        <v>62823300</v>
+        <v>62821800</v>
       </c>
       <c r="D7" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="8" spans="1:4">
@@ -2641,7 +2638,7 @@
         <v>60942100</v>
       </c>
       <c r="D8" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="9" spans="1:4">
@@ -2652,10 +2649,10 @@
         <v>328</v>
       </c>
       <c r="C9">
-        <v>58078200</v>
+        <v>58076500</v>
       </c>
       <c r="D9" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="10" spans="1:4">
@@ -2666,10 +2663,10 @@
         <v>329</v>
       </c>
       <c r="C10">
-        <v>58004600</v>
+        <v>58004500</v>
       </c>
       <c r="D10" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="11" spans="1:4">
@@ -2680,10 +2677,10 @@
         <v>330</v>
       </c>
       <c r="C11">
-        <v>49150000</v>
+        <v>49136200</v>
       </c>
       <c r="D11" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="12" spans="1:4">
@@ -2697,7 +2694,7 @@
         <v>38056400</v>
       </c>
       <c r="D12" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="13" spans="1:4">
@@ -2711,7 +2708,7 @@
         <v>37322000</v>
       </c>
       <c r="D13" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="14" spans="1:4">
@@ -2725,7 +2722,7 @@
         <v>34768700</v>
       </c>
       <c r="D14" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="15" spans="1:4">
@@ -2736,10 +2733,10 @@
         <v>334</v>
       </c>
       <c r="C15">
-        <v>30501400</v>
+        <v>30501200</v>
       </c>
       <c r="D15" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="16" spans="1:4">
@@ -2753,7 +2750,7 @@
         <v>26973800</v>
       </c>
       <c r="D16" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="17" spans="1:4">
@@ -2767,7 +2764,7 @@
         <v>25075600</v>
       </c>
       <c r="D17" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="18" spans="1:4">
@@ -2781,7 +2778,7 @@
         <v>24979900</v>
       </c>
       <c r="D18" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="19" spans="1:4">
@@ -2792,10 +2789,10 @@
         <v>338</v>
       </c>
       <c r="C19">
-        <v>24425900</v>
+        <v>24419400</v>
       </c>
       <c r="D19" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="20" spans="1:4">
@@ -2809,7 +2806,7 @@
         <v>24161300</v>
       </c>
       <c r="D20" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="21" spans="1:4">
@@ -2820,10 +2817,10 @@
         <v>340</v>
       </c>
       <c r="C21">
-        <v>23513400</v>
+        <v>23441600</v>
       </c>
       <c r="D21" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="22" spans="1:4">
@@ -2837,7 +2834,7 @@
         <v>19842500</v>
       </c>
       <c r="D22" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="23" spans="1:4">
@@ -2851,7 +2848,7 @@
         <v>18500200</v>
       </c>
       <c r="D23" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="24" spans="1:4">
@@ -2862,10 +2859,10 @@
         <v>343</v>
       </c>
       <c r="C24">
-        <v>17467500</v>
+        <v>17466500</v>
       </c>
       <c r="D24" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="25" spans="1:4">
@@ -2879,7 +2876,7 @@
         <v>15989200</v>
       </c>
       <c r="D25" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="26" spans="1:4">
@@ -2893,7 +2890,7 @@
         <v>15558800</v>
       </c>
       <c r="D26" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="27" spans="1:4">
@@ -2907,7 +2904,7 @@
         <v>15413000</v>
       </c>
       <c r="D27" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="28" spans="1:4">
@@ -2921,7 +2918,7 @@
         <v>15323400</v>
       </c>
       <c r="D28" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="29" spans="1:4">
@@ -2932,10 +2929,10 @@
         <v>348</v>
       </c>
       <c r="C29">
-        <v>15028400</v>
+        <v>15024800</v>
       </c>
       <c r="D29" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="30" spans="1:4">
@@ -2949,7 +2946,7 @@
         <v>14974900</v>
       </c>
       <c r="D30" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="31" spans="1:4">
@@ -2963,7 +2960,7 @@
         <v>13122800</v>
       </c>
       <c r="D31" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="32" spans="1:4">
@@ -2977,7 +2974,7 @@
         <v>12802800</v>
       </c>
       <c r="D32" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="33" spans="1:4">
@@ -2991,7 +2988,7 @@
         <v>12685300</v>
       </c>
       <c r="D33" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="34" spans="1:4">
@@ -3002,10 +2999,10 @@
         <v>353</v>
       </c>
       <c r="C34">
-        <v>12333500</v>
+        <v>12333300</v>
       </c>
       <c r="D34" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="35" spans="1:4">
@@ -3019,7 +3016,7 @@
         <v>12227800</v>
       </c>
       <c r="D35" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="36" spans="1:4">
@@ -3033,7 +3030,7 @@
         <v>11829600</v>
       </c>
       <c r="D36" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="37" spans="1:4">
@@ -3044,10 +3041,10 @@
         <v>356</v>
       </c>
       <c r="C37">
-        <v>11369900</v>
+        <v>11369400</v>
       </c>
       <c r="D37" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="38" spans="1:4">
@@ -3058,10 +3055,10 @@
         <v>357</v>
       </c>
       <c r="C38">
-        <v>11164000</v>
+        <v>11161000</v>
       </c>
       <c r="D38" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="39" spans="1:4">
@@ -3075,7 +3072,7 @@
         <v>11015500</v>
       </c>
       <c r="D39" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="40" spans="1:4">
@@ -3089,7 +3086,7 @@
         <v>10926300</v>
       </c>
       <c r="D40" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="41" spans="1:4">
@@ -3103,7 +3100,7 @@
         <v>10911500</v>
       </c>
       <c r="D41" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="42" spans="1:4">
@@ -3117,7 +3114,7 @@
         <v>10694300</v>
       </c>
       <c r="D42" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="43" spans="1:4">
@@ -3131,7 +3128,7 @@
         <v>10679100</v>
       </c>
       <c r="D43" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="44" spans="1:4">
@@ -3145,7 +3142,7 @@
         <v>10551500</v>
       </c>
       <c r="D44" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="45" spans="1:4">
@@ -3159,7 +3156,7 @@
         <v>10331000</v>
       </c>
       <c r="D45" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="46" spans="1:4">
@@ -3170,10 +3167,10 @@
         <v>365</v>
       </c>
       <c r="C46">
-        <v>10328800</v>
+        <v>10326400</v>
       </c>
       <c r="D46" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="47" spans="1:4">
@@ -3184,10 +3181,10 @@
         <v>366</v>
       </c>
       <c r="C47">
-        <v>10057500</v>
+        <v>10055500</v>
       </c>
       <c r="D47" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="48" spans="1:4">
@@ -3201,7 +3198,7 @@
         <v>9721600</v>
       </c>
       <c r="D48" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="49" spans="1:4">
@@ -3215,7 +3212,7 @@
         <v>9657500</v>
       </c>
       <c r="D49" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="50" spans="1:4">
@@ -3229,7 +3226,7 @@
         <v>8878500</v>
       </c>
       <c r="D50" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="51" spans="1:4">
@@ -3243,7 +3240,7 @@
         <v>8789300</v>
       </c>
       <c r="D51" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="52" spans="1:4">
@@ -3257,7 +3254,7 @@
         <v>8694900</v>
       </c>
       <c r="D52" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="53" spans="1:4">
@@ -3271,7 +3268,7 @@
         <v>8582900</v>
       </c>
       <c r="D53" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="54" spans="1:4">
@@ -3285,7 +3282,7 @@
         <v>8328500</v>
       </c>
       <c r="D54" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="55" spans="1:4">
@@ -3299,7 +3296,7 @@
         <v>8188000</v>
       </c>
       <c r="D55" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="56" spans="1:4">
@@ -3313,7 +3310,7 @@
         <v>8157400</v>
       </c>
       <c r="D56" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="57" spans="1:4">
@@ -3327,7 +3324,7 @@
         <v>7991700</v>
       </c>
       <c r="D57" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="58" spans="1:4">
@@ -3341,7 +3338,7 @@
         <v>7717100</v>
       </c>
       <c r="D58" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="59" spans="1:4">
@@ -3352,10 +3349,10 @@
         <v>378</v>
       </c>
       <c r="C59">
-        <v>7698100</v>
+        <v>7697100</v>
       </c>
       <c r="D59" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="60" spans="1:4">
@@ -3369,7 +3366,7 @@
         <v>7566100</v>
       </c>
       <c r="D60" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="61" spans="1:4">
@@ -3383,7 +3380,7 @@
         <v>7416700</v>
       </c>
       <c r="D61" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="62" spans="1:4">
@@ -3394,10 +3391,10 @@
         <v>381</v>
       </c>
       <c r="C62">
-        <v>7297700</v>
+        <v>7297400</v>
       </c>
       <c r="D62" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="63" spans="1:4">
@@ -3411,7 +3408,7 @@
         <v>7269600</v>
       </c>
       <c r="D63" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="64" spans="1:4">
@@ -3425,7 +3422,7 @@
         <v>7236400</v>
       </c>
       <c r="D64" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="65" spans="1:4">
@@ -3439,7 +3436,7 @@
         <v>6671300</v>
       </c>
       <c r="D65" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="66" spans="1:4">
@@ -3453,7 +3450,7 @@
         <v>6518700</v>
       </c>
       <c r="D66" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="67" spans="1:4">
@@ -3467,7 +3464,7 @@
         <v>6503500</v>
       </c>
       <c r="D67" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="68" spans="1:4">
@@ -3481,7 +3478,7 @@
         <v>6056900</v>
       </c>
       <c r="D68" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="69" spans="1:4">
@@ -3492,10 +3489,10 @@
         <v>388</v>
       </c>
       <c r="C69">
-        <v>6039300</v>
+        <v>6033700</v>
       </c>
       <c r="D69" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="70" spans="1:4">
@@ -3509,7 +3506,7 @@
         <v>5972700</v>
       </c>
       <c r="D70" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="71" spans="1:4">
@@ -3523,7 +3520,7 @@
         <v>5966400</v>
       </c>
       <c r="D71" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="72" spans="1:4">
@@ -3537,7 +3534,7 @@
         <v>5555100</v>
       </c>
       <c r="D72" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="73" spans="1:4">
@@ -3551,7 +3548,7 @@
         <v>5486400</v>
       </c>
       <c r="D73" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="74" spans="1:4">
@@ -3565,7 +3562,7 @@
         <v>5405000</v>
       </c>
       <c r="D74" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="75" spans="1:4">
@@ -3579,7 +3576,7 @@
         <v>5311100</v>
       </c>
       <c r="D75" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="76" spans="1:4">
@@ -3593,7 +3590,7 @@
         <v>5232500</v>
       </c>
       <c r="D76" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="77" spans="1:4">
@@ -3607,7 +3604,7 @@
         <v>5158200</v>
       </c>
       <c r="D77" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="78" spans="1:4">
@@ -3621,7 +3618,7 @@
         <v>5157000</v>
       </c>
       <c r="D78" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="79" spans="1:4">
@@ -3635,7 +3632,7 @@
         <v>4900000</v>
       </c>
       <c r="D79" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="80" spans="1:4">
@@ -3649,7 +3646,7 @@
         <v>4881500</v>
       </c>
       <c r="D80" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="81" spans="1:4">
@@ -3660,10 +3657,10 @@
         <v>400</v>
       </c>
       <c r="C81">
-        <v>4763800</v>
+        <v>4763700</v>
       </c>
       <c r="D81" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="82" spans="1:4">
@@ -3674,10 +3671,10 @@
         <v>401</v>
       </c>
       <c r="C82">
-        <v>4730600</v>
+        <v>4730200</v>
       </c>
       <c r="D82" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="83" spans="1:4">
@@ -3691,7 +3688,7 @@
         <v>4682000</v>
       </c>
       <c r="D83" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="84" spans="1:4">
@@ -3705,7 +3702,7 @@
         <v>4462300</v>
       </c>
       <c r="D84" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="85" spans="1:4">
@@ -3716,10 +3713,10 @@
         <v>404</v>
       </c>
       <c r="C85">
-        <v>4426100</v>
+        <v>4424100</v>
       </c>
       <c r="D85" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="86" spans="1:4">
@@ -3733,7 +3730,7 @@
         <v>4373100</v>
       </c>
       <c r="D86" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="87" spans="1:4">
@@ -3747,7 +3744,7 @@
         <v>4214200</v>
       </c>
       <c r="D87" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="88" spans="1:4">
@@ -3761,7 +3758,7 @@
         <v>4208100</v>
       </c>
       <c r="D88" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="89" spans="1:4">
@@ -3775,7 +3772,7 @@
         <v>4201500</v>
       </c>
       <c r="D89" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="90" spans="1:4">
@@ -3789,7 +3786,7 @@
         <v>4194500</v>
       </c>
       <c r="D90" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="91" spans="1:4">
@@ -3803,7 +3800,7 @@
         <v>4069600</v>
       </c>
       <c r="D91" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="92" spans="1:4">
@@ -3817,7 +3814,7 @@
         <v>3984900</v>
       </c>
       <c r="D92" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="93" spans="1:4">
@@ -3831,7 +3828,7 @@
         <v>3891400</v>
       </c>
       <c r="D93" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="94" spans="1:4">
@@ -3845,7 +3842,7 @@
         <v>3836700</v>
       </c>
       <c r="D94" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="95" spans="1:4">
@@ -3859,7 +3856,7 @@
         <v>3783800</v>
       </c>
       <c r="D95" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="96" spans="1:4">
@@ -3873,7 +3870,7 @@
         <v>3704500</v>
       </c>
       <c r="D96" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="97" spans="1:4">
@@ -3884,10 +3881,10 @@
         <v>416</v>
       </c>
       <c r="C97">
-        <v>3652700</v>
+        <v>3651600</v>
       </c>
       <c r="D97" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="98" spans="1:4">
@@ -3898,10 +3895,10 @@
         <v>417</v>
       </c>
       <c r="C98">
-        <v>3651600</v>
+        <v>3646700</v>
       </c>
       <c r="D98" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="99" spans="1:4">
@@ -3915,7 +3912,7 @@
         <v>3619300</v>
       </c>
       <c r="D99" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="100" spans="1:4">
@@ -3929,7 +3926,7 @@
         <v>3572600</v>
       </c>
       <c r="D100" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="101" spans="1:4">
@@ -3943,7 +3940,7 @@
         <v>3384700</v>
       </c>
       <c r="D101" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="102" spans="1:4">
@@ -3954,10 +3951,10 @@
         <v>421</v>
       </c>
       <c r="C102">
-        <v>3273500</v>
+        <v>3273300</v>
       </c>
       <c r="D102" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="103" spans="1:4">
@@ -3968,10 +3965,10 @@
         <v>422</v>
       </c>
       <c r="C103">
-        <v>3174900</v>
+        <v>3173900</v>
       </c>
       <c r="D103" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="104" spans="1:4">
@@ -3985,7 +3982,7 @@
         <v>2935500</v>
       </c>
       <c r="D104" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="105" spans="1:4">
@@ -3999,7 +3996,7 @@
         <v>2900500</v>
       </c>
       <c r="D105" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="106" spans="1:4">
@@ -4013,7 +4010,7 @@
         <v>2865100</v>
       </c>
       <c r="D106" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="107" spans="1:4">
@@ -4027,7 +4024,7 @@
         <v>2744500</v>
       </c>
       <c r="D107" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="108" spans="1:4">
@@ -4041,7 +4038,7 @@
         <v>2673900</v>
       </c>
       <c r="D108" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="109" spans="1:4">
@@ -4055,7 +4052,7 @@
         <v>2465700</v>
       </c>
       <c r="D109" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="110" spans="1:4">
@@ -4069,7 +4066,7 @@
         <v>2448900</v>
       </c>
       <c r="D110" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="111" spans="1:4">
@@ -4083,7 +4080,7 @@
         <v>2347200</v>
       </c>
       <c r="D111" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="112" spans="1:4">
@@ -4097,7 +4094,7 @@
         <v>2252400</v>
       </c>
       <c r="D112" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="113" spans="1:4">
@@ -4111,7 +4108,7 @@
         <v>2249100</v>
       </c>
       <c r="D113" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="114" spans="1:4">
@@ -4125,7 +4122,7 @@
         <v>2245400</v>
       </c>
       <c r="D114" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="115" spans="1:4">
@@ -4139,7 +4136,7 @@
         <v>2158600</v>
       </c>
       <c r="D115" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="116" spans="1:4">
@@ -4153,7 +4150,7 @@
         <v>2134800</v>
       </c>
       <c r="D116" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="117" spans="1:4">
@@ -4164,10 +4161,10 @@
         <v>436</v>
       </c>
       <c r="C117">
-        <v>2132900</v>
+        <v>2132600</v>
       </c>
       <c r="D117" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="118" spans="1:4">
@@ -4181,7 +4178,7 @@
         <v>2106600</v>
       </c>
       <c r="D118" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="119" spans="1:4">
@@ -4195,7 +4192,7 @@
         <v>1900600</v>
       </c>
       <c r="D119" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="120" spans="1:4">
@@ -4209,7 +4206,7 @@
         <v>1827900</v>
       </c>
       <c r="D120" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="121" spans="1:4">
@@ -4223,7 +4220,7 @@
         <v>1821600</v>
       </c>
       <c r="D121" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="122" spans="1:4">
@@ -4237,7 +4234,7 @@
         <v>1810100</v>
       </c>
       <c r="D122" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="123" spans="1:4">
@@ -4251,7 +4248,7 @@
         <v>1776200</v>
       </c>
       <c r="D123" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="124" spans="1:4">
@@ -4265,7 +4262,7 @@
         <v>1771300</v>
       </c>
       <c r="D124" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="125" spans="1:4">
@@ -4279,7 +4276,7 @@
         <v>1755500</v>
       </c>
       <c r="D125" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="126" spans="1:4">
@@ -4293,7 +4290,7 @@
         <v>1715200</v>
       </c>
       <c r="D126" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="127" spans="1:4">
@@ -4307,7 +4304,7 @@
         <v>1663800</v>
       </c>
       <c r="D127" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="128" spans="1:4">
@@ -4318,10 +4315,10 @@
         <v>447</v>
       </c>
       <c r="C128">
-        <v>1633500</v>
+        <v>1633200</v>
       </c>
       <c r="D128" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="129" spans="1:4">
@@ -4332,10 +4329,10 @@
         <v>448</v>
       </c>
       <c r="C129">
-        <v>1629800</v>
+        <v>1624500</v>
       </c>
       <c r="D129" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="130" spans="1:4">
@@ -4346,10 +4343,10 @@
         <v>449</v>
       </c>
       <c r="C130">
-        <v>1624500</v>
+        <v>1600900</v>
       </c>
       <c r="D130" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="131" spans="1:4">
@@ -4360,10 +4357,10 @@
         <v>450</v>
       </c>
       <c r="C131">
-        <v>1600900</v>
+        <v>1589800</v>
       </c>
       <c r="D131" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="132" spans="1:4">
@@ -4377,7 +4374,7 @@
         <v>1567400</v>
       </c>
       <c r="D132" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="133" spans="1:4">
@@ -4391,12 +4388,12 @@
         <v>1533600</v>
       </c>
       <c r="D133" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="134" spans="1:4">
       <c r="A134" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="B134" t="s">
         <v>453</v>
@@ -4405,7 +4402,7 @@
         <v>1526500</v>
       </c>
       <c r="D134" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="135" spans="1:4">
@@ -4419,7 +4416,7 @@
         <v>1486100</v>
       </c>
       <c r="D135" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="136" spans="1:4">
@@ -4433,7 +4430,7 @@
         <v>1470400</v>
       </c>
       <c r="D136" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="137" spans="1:4">
@@ -4447,7 +4444,7 @@
         <v>1452100</v>
       </c>
       <c r="D137" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="138" spans="1:4">
@@ -4461,7 +4458,7 @@
         <v>1392000</v>
       </c>
       <c r="D138" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="139" spans="1:4">
@@ -4475,7 +4472,7 @@
         <v>1367300</v>
       </c>
       <c r="D139" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="140" spans="1:4">
@@ -4489,7 +4486,7 @@
         <v>1334200</v>
       </c>
       <c r="D140" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="141" spans="1:4">
@@ -4503,7 +4500,7 @@
         <v>1294600</v>
       </c>
       <c r="D141" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="142" spans="1:4">
@@ -4517,7 +4514,7 @@
         <v>1254600</v>
       </c>
       <c r="D142" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="143" spans="1:4">
@@ -4531,7 +4528,7 @@
         <v>1213700</v>
       </c>
       <c r="D143" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="144" spans="1:4">
@@ -4545,7 +4542,7 @@
         <v>1200400</v>
       </c>
       <c r="D144" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="145" spans="1:4">
@@ -4556,10 +4553,10 @@
         <v>464</v>
       </c>
       <c r="C145">
-        <v>1177000</v>
+        <v>1176900</v>
       </c>
       <c r="D145" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="146" spans="1:4">
@@ -4573,7 +4570,7 @@
         <v>1176800</v>
       </c>
       <c r="D146" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="147" spans="1:4">
@@ -4587,7 +4584,7 @@
         <v>1176700</v>
       </c>
       <c r="D147" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="148" spans="1:4">
@@ -4601,7 +4598,7 @@
         <v>1110800</v>
       </c>
       <c r="D148" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="149" spans="1:4">
@@ -4615,7 +4612,7 @@
         <v>1081500</v>
       </c>
       <c r="D149" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="150" spans="1:4">
@@ -4629,7 +4626,7 @@
         <v>1035200</v>
       </c>
       <c r="D150" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="151" spans="1:4">
@@ -4643,7 +4640,7 @@
         <v>990000</v>
       </c>
       <c r="D151" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="152" spans="1:4">
@@ -4657,7 +4654,7 @@
         <v>945500</v>
       </c>
       <c r="D152" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="153" spans="1:4">
@@ -4671,7 +4668,7 @@
         <v>900300</v>
       </c>
       <c r="D153" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="154" spans="1:4">
@@ -4685,7 +4682,7 @@
         <v>896100</v>
       </c>
       <c r="D154" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="155" spans="1:4">
@@ -4699,7 +4696,7 @@
         <v>867400</v>
       </c>
       <c r="D155" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="156" spans="1:4">
@@ -4713,7 +4710,7 @@
         <v>858600</v>
       </c>
       <c r="D156" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="157" spans="1:4">
@@ -4727,7 +4724,7 @@
         <v>823400</v>
       </c>
       <c r="D157" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="158" spans="1:4">
@@ -4741,7 +4738,7 @@
         <v>813400</v>
       </c>
       <c r="D158" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="159" spans="1:4">
@@ -4755,7 +4752,7 @@
         <v>799500</v>
       </c>
       <c r="D159" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="160" spans="1:4">
@@ -4769,7 +4766,7 @@
         <v>771600</v>
       </c>
       <c r="D160" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="161" spans="1:4">
@@ -4783,7 +4780,7 @@
         <v>760200</v>
       </c>
       <c r="D161" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="162" spans="1:4">
@@ -4797,7 +4794,7 @@
         <v>752600</v>
       </c>
       <c r="D162" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="163" spans="1:4">
@@ -4811,7 +4808,7 @@
         <v>752300</v>
       </c>
       <c r="D163" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="164" spans="1:4">
@@ -4825,7 +4822,7 @@
         <v>742100</v>
       </c>
       <c r="D164" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="165" spans="1:4">
@@ -4839,7 +4836,7 @@
         <v>731600</v>
       </c>
       <c r="D165" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="166" spans="1:4">
@@ -4853,7 +4850,7 @@
         <v>699400</v>
       </c>
       <c r="D166" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="167" spans="1:4">
@@ -4867,7 +4864,7 @@
         <v>690500</v>
       </c>
       <c r="D167" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="168" spans="1:4">
@@ -4881,7 +4878,7 @@
         <v>676400</v>
       </c>
       <c r="D168" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="169" spans="1:4">
@@ -4895,7 +4892,7 @@
         <v>655400</v>
       </c>
       <c r="D169" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="170" spans="1:4">
@@ -4909,7 +4906,7 @@
         <v>642700</v>
       </c>
       <c r="D170" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="171" spans="1:4">
@@ -4923,7 +4920,7 @@
         <v>632500</v>
       </c>
       <c r="D171" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="172" spans="1:4">
@@ -4937,7 +4934,7 @@
         <v>618000</v>
       </c>
       <c r="D172" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="173" spans="1:4">
@@ -4951,7 +4948,7 @@
         <v>531900</v>
       </c>
       <c r="D173" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="174" spans="1:4">
@@ -4965,7 +4962,7 @@
         <v>509200</v>
       </c>
       <c r="D174" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="175" spans="1:4">
@@ -4979,7 +4976,7 @@
         <v>504100</v>
       </c>
       <c r="D175" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="176" spans="1:4">
@@ -4993,7 +4990,7 @@
         <v>475800</v>
       </c>
       <c r="D176" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="177" spans="1:4">
@@ -5007,7 +5004,7 @@
         <v>438300</v>
       </c>
       <c r="D177" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="178" spans="1:4">
@@ -5021,7 +5018,7 @@
         <v>438200</v>
       </c>
       <c r="D178" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="179" spans="1:4">
@@ -5035,7 +5032,7 @@
         <v>422000</v>
       </c>
       <c r="D179" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="180" spans="1:4">
@@ -5049,7 +5046,7 @@
         <v>417600</v>
       </c>
       <c r="D180" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="181" spans="1:4">
@@ -5063,7 +5060,7 @@
         <v>406800</v>
       </c>
       <c r="D181" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="182" spans="1:4">
@@ -5077,7 +5074,7 @@
         <v>400700</v>
       </c>
       <c r="D182" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="183" spans="1:4">
@@ -5091,7 +5088,7 @@
         <v>400200</v>
       </c>
       <c r="D183" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="184" spans="1:4">
@@ -5105,7 +5102,7 @@
         <v>383300</v>
       </c>
       <c r="D184" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="185" spans="1:4">
@@ -5119,7 +5116,7 @@
         <v>371300</v>
       </c>
       <c r="D185" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="186" spans="1:4">
@@ -5133,7 +5130,7 @@
         <v>362400</v>
       </c>
       <c r="D186" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="187" spans="1:4">
@@ -5147,7 +5144,7 @@
         <v>347300</v>
       </c>
       <c r="D187" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="188" spans="1:4">
@@ -5161,7 +5158,7 @@
         <v>325400</v>
       </c>
       <c r="D188" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="189" spans="1:4">
@@ -5175,7 +5172,7 @@
         <v>317000</v>
       </c>
       <c r="D189" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="190" spans="1:4">
@@ -5189,7 +5186,7 @@
         <v>313300</v>
       </c>
       <c r="D190" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="191" spans="1:4">
@@ -5203,7 +5200,7 @@
         <v>307200</v>
       </c>
       <c r="D191" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="192" spans="1:4">
@@ -5217,7 +5214,7 @@
         <v>296400</v>
       </c>
       <c r="D192" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="193" spans="1:4">
@@ -5231,7 +5228,7 @@
         <v>295000</v>
       </c>
       <c r="D193" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="194" spans="1:4">
@@ -5245,7 +5242,7 @@
         <v>292200</v>
       </c>
       <c r="D194" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="195" spans="1:4">
@@ -5259,7 +5256,7 @@
         <v>291600</v>
       </c>
       <c r="D195" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="196" spans="1:4">
@@ -5273,7 +5270,7 @@
         <v>280100</v>
       </c>
       <c r="D196" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="197" spans="1:4">
@@ -5287,7 +5284,7 @@
         <v>263200</v>
       </c>
       <c r="D197" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="198" spans="1:4">
@@ -5301,7 +5298,7 @@
         <v>260400</v>
       </c>
       <c r="D198" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="199" spans="1:4">
@@ -5315,7 +5312,7 @@
         <v>257700</v>
       </c>
       <c r="D199" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="200" spans="1:4">
@@ -5329,7 +5326,7 @@
         <v>254400</v>
       </c>
       <c r="D200" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="201" spans="1:4">
@@ -5343,7 +5340,7 @@
         <v>251100</v>
       </c>
       <c r="D201" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="202" spans="1:4">
@@ -5357,7 +5354,7 @@
         <v>228100</v>
       </c>
       <c r="D202" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="203" spans="1:4">
@@ -5371,7 +5368,7 @@
         <v>200800</v>
       </c>
       <c r="D203" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="204" spans="1:4">
@@ -5385,7 +5382,7 @@
         <v>200000</v>
       </c>
       <c r="D204" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="205" spans="1:4">
@@ -5399,7 +5396,7 @@
         <v>196500</v>
       </c>
       <c r="D205" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="206" spans="1:4">
@@ -5413,7 +5410,7 @@
         <v>196300</v>
       </c>
       <c r="D206" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="207" spans="1:4">
@@ -5427,7 +5424,7 @@
         <v>195400</v>
       </c>
       <c r="D207" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="208" spans="1:4">
@@ -5441,7 +5438,7 @@
         <v>177200</v>
       </c>
       <c r="D208" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="209" spans="1:4">
@@ -5455,7 +5452,7 @@
         <v>176400</v>
       </c>
       <c r="D209" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="210" spans="1:4">
@@ -5469,7 +5466,7 @@
         <v>172000</v>
       </c>
       <c r="D210" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="211" spans="1:4">
@@ -5483,7 +5480,7 @@
         <v>163900</v>
       </c>
       <c r="D211" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="212" spans="1:4">
@@ -5497,7 +5494,7 @@
         <v>163200</v>
       </c>
       <c r="D212" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="213" spans="1:4">
@@ -5511,7 +5508,7 @@
         <v>159800</v>
       </c>
       <c r="D213" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="214" spans="1:4">
@@ -5525,7 +5522,7 @@
         <v>159500</v>
       </c>
       <c r="D214" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="215" spans="1:4">
@@ -5539,7 +5536,7 @@
         <v>153000</v>
       </c>
       <c r="D215" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="216" spans="1:4">
@@ -5553,7 +5550,7 @@
         <v>152500</v>
       </c>
       <c r="D216" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="217" spans="1:4">
@@ -5567,7 +5564,7 @@
         <v>148900</v>
       </c>
       <c r="D217" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="218" spans="1:4">
@@ -5581,7 +5578,7 @@
         <v>145700</v>
       </c>
       <c r="D218" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="219" spans="1:4">
@@ -5595,7 +5592,7 @@
         <v>143500</v>
       </c>
       <c r="D219" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="220" spans="1:4">
@@ -5609,7 +5606,7 @@
         <v>137800</v>
       </c>
       <c r="D220" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="221" spans="1:4">
@@ -5623,7 +5620,7 @@
         <v>132400</v>
       </c>
       <c r="D221" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="222" spans="1:4">
@@ -5637,7 +5634,7 @@
         <v>108500</v>
       </c>
       <c r="D222" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="223" spans="1:4">
@@ -5648,10 +5645,10 @@
         <v>542</v>
       </c>
       <c r="C223">
-        <v>101500</v>
+        <v>101300</v>
       </c>
       <c r="D223" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="224" spans="1:4">
@@ -5665,7 +5662,7 @@
         <v>98000</v>
       </c>
       <c r="D224" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="225" spans="1:4">
@@ -5679,7 +5676,7 @@
         <v>97100</v>
       </c>
       <c r="D225" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="226" spans="1:4">
@@ -5693,7 +5690,7 @@
         <v>74100</v>
       </c>
       <c r="D226" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="227" spans="1:4">
@@ -5707,7 +5704,7 @@
         <v>66400</v>
       </c>
       <c r="D227" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="228" spans="1:4">
@@ -5721,7 +5718,7 @@
         <v>64900</v>
       </c>
       <c r="D228" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="229" spans="1:4">
@@ -5732,10 +5729,10 @@
         <v>548</v>
       </c>
       <c r="C229">
-        <v>63900</v>
+        <v>62700</v>
       </c>
       <c r="D229" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="230" spans="1:4">
@@ -5749,7 +5746,7 @@
         <v>61700</v>
       </c>
       <c r="D230" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="231" spans="1:4">
@@ -5763,7 +5760,7 @@
         <v>59900</v>
       </c>
       <c r="D231" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="232" spans="1:4">
@@ -5777,7 +5774,7 @@
         <v>58100</v>
       </c>
       <c r="D232" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="233" spans="1:4">
@@ -5791,7 +5788,7 @@
         <v>53700</v>
       </c>
       <c r="D233" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="234" spans="1:4">
@@ -5805,7 +5802,7 @@
         <v>53300</v>
       </c>
       <c r="D234" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="235" spans="1:4">
@@ -5819,7 +5816,7 @@
         <v>53300</v>
       </c>
       <c r="D235" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="236" spans="1:4">
@@ -5833,7 +5830,7 @@
         <v>53100</v>
       </c>
       <c r="D236" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="237" spans="1:4">
@@ -5847,7 +5844,7 @@
         <v>50400</v>
       </c>
       <c r="D237" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="238" spans="1:4">
@@ -5858,15 +5855,15 @@
         <v>557</v>
       </c>
       <c r="C238">
-        <v>48100</v>
+        <v>47500</v>
       </c>
       <c r="D238" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="239" spans="1:4">
       <c r="A239" t="s">
-        <v>48</v>
+        <v>219</v>
       </c>
       <c r="B239" t="s">
         <v>558</v>
@@ -5875,12 +5872,12 @@
         <v>47200</v>
       </c>
       <c r="D239" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="240" spans="1:4">
       <c r="A240" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="B240" t="s">
         <v>559</v>
@@ -5889,12 +5886,12 @@
         <v>44600</v>
       </c>
       <c r="D240" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="241" spans="1:4">
       <c r="A241" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="B241" t="s">
         <v>560</v>
@@ -5903,7 +5900,7 @@
         <v>42400</v>
       </c>
       <c r="D241" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="242" spans="1:4">
@@ -5917,7 +5914,7 @@
         <v>41900</v>
       </c>
       <c r="D242" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="243" spans="1:4">
@@ -5931,12 +5928,12 @@
         <v>40900</v>
       </c>
       <c r="D243" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="244" spans="1:4">
       <c r="A244" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="B244" t="s">
         <v>563</v>
@@ -5945,12 +5942,12 @@
         <v>35900</v>
       </c>
       <c r="D244" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="245" spans="1:4">
       <c r="A245" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="B245" t="s">
         <v>564</v>
@@ -5959,12 +5956,12 @@
         <v>35400</v>
       </c>
       <c r="D245" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="246" spans="1:4">
       <c r="A246" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="B246" t="s">
         <v>565</v>
@@ -5973,7 +5970,7 @@
         <v>34100</v>
       </c>
       <c r="D246" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="247" spans="1:4">
@@ -5987,7 +5984,7 @@
         <v>33100</v>
       </c>
       <c r="D247" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="248" spans="1:4">
@@ -6001,12 +5998,12 @@
         <v>32200</v>
       </c>
       <c r="D248" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="249" spans="1:4">
       <c r="A249" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="B249" t="s">
         <v>568</v>
@@ -6015,12 +6012,12 @@
         <v>30400</v>
       </c>
       <c r="D249" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="250" spans="1:4">
       <c r="A250" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="B250" t="s">
         <v>569</v>
@@ -6029,26 +6026,26 @@
         <v>28400</v>
       </c>
       <c r="D250" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="251" spans="1:4">
       <c r="A251" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="B251" t="s">
         <v>570</v>
       </c>
       <c r="C251">
-        <v>27800</v>
+        <v>27500</v>
       </c>
       <c r="D251" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="252" spans="1:4">
       <c r="A252" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="B252" t="s">
         <v>571</v>
@@ -6057,7 +6054,7 @@
         <v>27000</v>
       </c>
       <c r="D252" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="253" spans="1:4">
@@ -6071,12 +6068,12 @@
         <v>25600</v>
       </c>
       <c r="D253" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="254" spans="1:4">
       <c r="A254" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="B254" t="s">
         <v>573</v>
@@ -6085,12 +6082,12 @@
         <v>24000</v>
       </c>
       <c r="D254" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="255" spans="1:4">
       <c r="A255" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="B255" t="s">
         <v>574</v>
@@ -6099,12 +6096,12 @@
         <v>22800</v>
       </c>
       <c r="D255" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="256" spans="1:4">
       <c r="A256" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="B256" t="s">
         <v>575</v>
@@ -6113,12 +6110,12 @@
         <v>16200</v>
       </c>
       <c r="D256" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="257" spans="1:4">
       <c r="A257" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="B257" t="s">
         <v>576</v>
@@ -6127,12 +6124,12 @@
         <v>15300</v>
       </c>
       <c r="D257" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="258" spans="1:4">
       <c r="A258" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="B258" t="s">
         <v>577</v>
@@ -6141,7 +6138,7 @@
         <v>15300</v>
       </c>
       <c r="D258" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="259" spans="1:4">
@@ -6155,7 +6152,7 @@
         <v>15100</v>
       </c>
       <c r="D259" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="260" spans="1:4">
@@ -6169,7 +6166,7 @@
         <v>14900</v>
       </c>
       <c r="D260" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="261" spans="1:4">
@@ -6183,12 +6180,12 @@
         <v>14200</v>
       </c>
       <c r="D261" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="262" spans="1:4">
       <c r="A262" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="B262" t="s">
         <v>581</v>
@@ -6197,12 +6194,12 @@
         <v>13300</v>
       </c>
       <c r="D262" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="263" spans="1:4">
       <c r="A263" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="B263" t="s">
         <v>582</v>
@@ -6211,7 +6208,7 @@
         <v>13300</v>
       </c>
       <c r="D263" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="264" spans="1:4">
@@ -6225,12 +6222,12 @@
         <v>13100</v>
       </c>
       <c r="D264" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="265" spans="1:4">
       <c r="A265" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="B265" t="s">
         <v>584</v>
@@ -6239,12 +6236,12 @@
         <v>11500</v>
       </c>
       <c r="D265" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="266" spans="1:4">
       <c r="A266" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="B266" t="s">
         <v>585</v>
@@ -6253,12 +6250,12 @@
         <v>11200</v>
       </c>
       <c r="D266" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="267" spans="1:4">
       <c r="A267" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="B267" t="s">
         <v>586</v>
@@ -6267,12 +6264,12 @@
         <v>10800</v>
       </c>
       <c r="D267" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="268" spans="1:4">
       <c r="A268" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="B268" t="s">
         <v>587</v>
@@ -6281,7 +6278,7 @@
         <v>10700</v>
       </c>
       <c r="D268" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="269" spans="1:4">
@@ -6295,12 +6292,12 @@
         <v>8800</v>
       </c>
       <c r="D269" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="270" spans="1:4">
       <c r="A270" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="B270" t="s">
         <v>589</v>
@@ -6309,12 +6306,12 @@
         <v>8600</v>
       </c>
       <c r="D270" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="271" spans="1:4">
       <c r="A271" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="B271" t="s">
         <v>590</v>
@@ -6323,12 +6320,12 @@
         <v>8100</v>
       </c>
       <c r="D271" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="272" spans="1:4">
       <c r="A272" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="B272" t="s">
         <v>591</v>
@@ -6337,12 +6334,12 @@
         <v>8000</v>
       </c>
       <c r="D272" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="273" spans="1:4">
       <c r="A273" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="B273" t="s">
         <v>592</v>
@@ -6351,7 +6348,7 @@
         <v>7000</v>
       </c>
       <c r="D273" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="274" spans="1:4">
@@ -6365,12 +6362,12 @@
         <v>6000</v>
       </c>
       <c r="D274" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="275" spans="1:4">
       <c r="A275" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="B275" t="s">
         <v>594</v>
@@ -6379,12 +6376,12 @@
         <v>5900</v>
       </c>
       <c r="D275" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="276" spans="1:4">
       <c r="A276" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="B276" t="s">
         <v>595</v>
@@ -6393,12 +6390,12 @@
         <v>5800</v>
       </c>
       <c r="D276" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="277" spans="1:4">
       <c r="A277" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="B277" t="s">
         <v>596</v>
@@ -6407,7 +6404,7 @@
         <v>5500</v>
       </c>
       <c r="D277" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="278" spans="1:4">
@@ -6421,12 +6418,12 @@
         <v>5200</v>
       </c>
       <c r="D278" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="279" spans="1:4">
       <c r="A279" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="B279" t="s">
         <v>598</v>
@@ -6435,12 +6432,12 @@
         <v>5200</v>
       </c>
       <c r="D279" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="280" spans="1:4">
       <c r="A280" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="B280" t="s">
         <v>599</v>
@@ -6449,12 +6446,12 @@
         <v>5000</v>
       </c>
       <c r="D280" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="281" spans="1:4">
       <c r="A281" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="B281" t="s">
         <v>600</v>
@@ -6463,12 +6460,12 @@
         <v>4900</v>
       </c>
       <c r="D281" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="282" spans="1:4">
       <c r="A282" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="B282" t="s">
         <v>601</v>
@@ -6477,7 +6474,7 @@
         <v>4700</v>
       </c>
       <c r="D282" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="283" spans="1:4">
@@ -6491,12 +6488,12 @@
         <v>4400</v>
       </c>
       <c r="D283" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="284" spans="1:4">
       <c r="A284" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="B284" t="s">
         <v>603</v>
@@ -6505,12 +6502,12 @@
         <v>4400</v>
       </c>
       <c r="D284" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="285" spans="1:4">
       <c r="A285" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="B285" t="s">
         <v>604</v>
@@ -6519,7 +6516,7 @@
         <v>4200</v>
       </c>
       <c r="D285" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="286" spans="1:4">
@@ -6533,12 +6530,12 @@
         <v>4000</v>
       </c>
       <c r="D286" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="287" spans="1:4">
       <c r="A287" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="B287" t="s">
         <v>606</v>
@@ -6547,12 +6544,12 @@
         <v>4000</v>
       </c>
       <c r="D287" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="288" spans="1:4">
       <c r="A288" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="B288" t="s">
         <v>607</v>
@@ -6561,12 +6558,12 @@
         <v>3900</v>
       </c>
       <c r="D288" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="289" spans="1:4">
       <c r="A289" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="B289" t="s">
         <v>608</v>
@@ -6575,7 +6572,7 @@
         <v>3800</v>
       </c>
       <c r="D289" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="290" spans="1:4">
@@ -6589,7 +6586,7 @@
         <v>3700</v>
       </c>
       <c r="D290" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="291" spans="1:4">
@@ -6603,12 +6600,12 @@
         <v>3600</v>
       </c>
       <c r="D291" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="292" spans="1:4">
       <c r="A292" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="B292" t="s">
         <v>611</v>
@@ -6617,12 +6614,12 @@
         <v>3500</v>
       </c>
       <c r="D292" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="293" spans="1:4">
       <c r="A293" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="B293" t="s">
         <v>612</v>
@@ -6631,12 +6628,12 @@
         <v>3500</v>
       </c>
       <c r="D293" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="294" spans="1:4">
       <c r="A294" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="B294" t="s">
         <v>613</v>
@@ -6645,12 +6642,12 @@
         <v>3400</v>
       </c>
       <c r="D294" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="295" spans="1:4">
       <c r="A295" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="B295" t="s">
         <v>614</v>
@@ -6659,7 +6656,7 @@
         <v>3300</v>
       </c>
       <c r="D295" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="296" spans="1:4">
@@ -6673,7 +6670,7 @@
         <v>3100</v>
       </c>
       <c r="D296" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="297" spans="1:4">
@@ -6687,12 +6684,12 @@
         <v>2900</v>
       </c>
       <c r="D297" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="298" spans="1:4">
       <c r="A298" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="B298" t="s">
         <v>617</v>
@@ -6701,12 +6698,12 @@
         <v>2800</v>
       </c>
       <c r="D298" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="299" spans="1:4">
       <c r="A299" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="B299" t="s">
         <v>618</v>
@@ -6715,12 +6712,12 @@
         <v>2700</v>
       </c>
       <c r="D299" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="300" spans="1:4">
       <c r="A300" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="B300" t="s">
         <v>619</v>
@@ -6729,12 +6726,12 @@
         <v>2700</v>
       </c>
       <c r="D300" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="301" spans="1:4">
       <c r="A301" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="B301" t="s">
         <v>620</v>
@@ -6743,12 +6740,12 @@
         <v>2700</v>
       </c>
       <c r="D301" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="302" spans="1:4">
       <c r="A302" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="B302" t="s">
         <v>621</v>
@@ -6757,40 +6754,40 @@
         <v>2500</v>
       </c>
       <c r="D302" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="303" spans="1:4">
       <c r="A303" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="B303" t="s">
-        <v>622</v>
+        <v>261</v>
       </c>
       <c r="C303">
         <v>2400</v>
       </c>
       <c r="D303" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="304" spans="1:4">
       <c r="A304" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="B304" t="s">
-        <v>261</v>
+        <v>622</v>
       </c>
       <c r="C304">
-        <v>2400</v>
+        <v>2300</v>
       </c>
       <c r="D304" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="305" spans="1:4">
       <c r="A305" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="B305" t="s">
         <v>623</v>
@@ -6799,12 +6796,12 @@
         <v>2300</v>
       </c>
       <c r="D305" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="306" spans="1:4">
       <c r="A306" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="B306" t="s">
         <v>624</v>
@@ -6813,12 +6810,12 @@
         <v>2300</v>
       </c>
       <c r="D306" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="307" spans="1:4">
       <c r="A307" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="B307" t="s">
         <v>625</v>
@@ -6827,12 +6824,12 @@
         <v>2300</v>
       </c>
       <c r="D307" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="308" spans="1:4">
       <c r="A308" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="B308" t="s">
         <v>626</v>
@@ -6841,7 +6838,7 @@
         <v>2200</v>
       </c>
       <c r="D308" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="309" spans="1:4">
@@ -6855,12 +6852,12 @@
         <v>2100</v>
       </c>
       <c r="D309" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="310" spans="1:4">
       <c r="A310" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="B310" t="s">
         <v>628</v>
@@ -6869,12 +6866,12 @@
         <v>2000</v>
       </c>
       <c r="D310" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="311" spans="1:4">
       <c r="A311" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="B311" t="s">
         <v>629</v>
@@ -6883,7 +6880,7 @@
         <v>1800</v>
       </c>
       <c r="D311" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="312" spans="1:4">
@@ -6897,12 +6894,12 @@
         <v>1700</v>
       </c>
       <c r="D312" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="313" spans="1:4">
       <c r="A313" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="B313" t="s">
         <v>631</v>
@@ -6911,12 +6908,12 @@
         <v>1600</v>
       </c>
       <c r="D313" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="314" spans="1:4">
       <c r="A314" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="B314" t="s">
         <v>632</v>
@@ -6925,12 +6922,12 @@
         <v>1600</v>
       </c>
       <c r="D314" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="315" spans="1:4">
       <c r="A315" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="B315" t="s">
         <v>633</v>
@@ -6939,12 +6936,12 @@
         <v>1600</v>
       </c>
       <c r="D315" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="316" spans="1:4">
       <c r="A316" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="B316" t="s">
         <v>634</v>
@@ -6953,12 +6950,12 @@
         <v>1300</v>
       </c>
       <c r="D316" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="317" spans="1:4">
       <c r="A317" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="B317" t="s">
         <v>635</v>
@@ -6967,12 +6964,12 @@
         <v>1100</v>
       </c>
       <c r="D317" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="318" spans="1:4">
       <c r="A318" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="B318" t="s">
         <v>636</v>
@@ -6981,12 +6978,12 @@
         <v>1000</v>
       </c>
       <c r="D318" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="319" spans="1:4">
       <c r="A319" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="B319" t="s">
         <v>637</v>
@@ -6995,12 +6992,12 @@
         <v>900</v>
       </c>
       <c r="D319" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="320" spans="1:4">
       <c r="A320" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="B320" t="s">
         <v>638</v>
@@ -7009,26 +7006,26 @@
         <v>900</v>
       </c>
       <c r="D320" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="321" spans="1:4">
       <c r="A321" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="B321" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="C321">
         <v>900</v>
       </c>
       <c r="D321" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="322" spans="1:4">
       <c r="A322" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="B322" t="s">
         <v>639</v>
@@ -7037,12 +7034,12 @@
         <v>800</v>
       </c>
       <c r="D322" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="323" spans="1:4">
       <c r="A323" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="B323" t="s">
         <v>640</v>
@@ -7051,12 +7048,12 @@
         <v>800</v>
       </c>
       <c r="D323" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="324" spans="1:4">
       <c r="A324" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="B324" t="s">
         <v>641</v>
@@ -7065,12 +7062,12 @@
         <v>700</v>
       </c>
       <c r="D324" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="325" spans="1:4">
       <c r="A325" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="B325" t="s">
         <v>642</v>
@@ -7079,12 +7076,12 @@
         <v>600</v>
       </c>
       <c r="D325" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="326" spans="1:4">
       <c r="A326" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="B326" t="s">
         <v>643</v>
@@ -7093,12 +7090,12 @@
         <v>600</v>
       </c>
       <c r="D326" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="327" spans="1:4">
       <c r="A327" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="B327" t="s">
         <v>644</v>
@@ -7107,12 +7104,12 @@
         <v>600</v>
       </c>
       <c r="D327" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="328" spans="1:4">
       <c r="A328" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="B328" t="s">
         <v>645</v>
@@ -7121,12 +7118,12 @@
         <v>600</v>
       </c>
       <c r="D328" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="329" spans="1:4">
       <c r="A329" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="B329" t="s">
         <v>646</v>
@@ -7135,12 +7132,12 @@
         <v>500</v>
       </c>
       <c r="D329" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="330" spans="1:4">
       <c r="A330" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="B330" t="s">
         <v>647</v>
@@ -7149,12 +7146,12 @@
         <v>500</v>
       </c>
       <c r="D330" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="331" spans="1:4">
       <c r="A331" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="B331" t="s">
         <v>648</v>
@@ -7163,12 +7160,12 @@
         <v>500</v>
       </c>
       <c r="D331" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="332" spans="1:4">
       <c r="A332" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="B332" t="s">
         <v>649</v>
@@ -7177,7 +7174,7 @@
         <v>400</v>
       </c>
       <c r="D332" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="333" spans="1:4">
@@ -7191,12 +7188,12 @@
         <v>400</v>
       </c>
       <c r="D333" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="334" spans="1:4">
       <c r="A334" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="B334" t="s">
         <v>651</v>
@@ -7205,12 +7202,12 @@
         <v>400</v>
       </c>
       <c r="D334" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="335" spans="1:4">
       <c r="A335" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="B335" t="s">
         <v>652</v>
@@ -7219,12 +7216,12 @@
         <v>400</v>
       </c>
       <c r="D335" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="336" spans="1:4">
       <c r="A336" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="B336" t="s">
         <v>653</v>
@@ -7233,7 +7230,7 @@
         <v>300</v>
       </c>
       <c r="D336" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="337" spans="1:4">
@@ -7247,12 +7244,12 @@
         <v>300</v>
       </c>
       <c r="D337" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="338" spans="1:4">
       <c r="A338" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="B338" t="s">
         <v>655</v>
@@ -7261,12 +7258,12 @@
         <v>300</v>
       </c>
       <c r="D338" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="339" spans="1:4">
       <c r="A339" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="B339" t="s">
         <v>656</v>
@@ -7275,12 +7272,12 @@
         <v>300</v>
       </c>
       <c r="D339" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="340" spans="1:4">
       <c r="A340" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="B340" t="s">
         <v>657</v>
@@ -7289,12 +7286,12 @@
         <v>200</v>
       </c>
       <c r="D340" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="341" spans="1:4">
       <c r="A341" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="B341" t="s">
         <v>658</v>
@@ -7303,12 +7300,12 @@
         <v>200</v>
       </c>
       <c r="D341" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="342" spans="1:4">
       <c r="A342" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="B342" t="s">
         <v>659</v>
@@ -7317,12 +7314,12 @@
         <v>200</v>
       </c>
       <c r="D342" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="343" spans="1:4">
       <c r="A343" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="B343" t="s">
         <v>660</v>
@@ -7331,12 +7328,12 @@
         <v>200</v>
       </c>
       <c r="D343" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="344" spans="1:4">
       <c r="A344" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="B344" t="s">
         <v>661</v>
@@ -7345,7 +7342,7 @@
         <v>200</v>
       </c>
       <c r="D344" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="345" spans="1:4">
@@ -7359,12 +7356,12 @@
         <v>200</v>
       </c>
       <c r="D345" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="346" spans="1:4">
       <c r="A346" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="B346" t="s">
         <v>663</v>
@@ -7373,12 +7370,12 @@
         <v>200</v>
       </c>
       <c r="D346" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="347" spans="1:4">
       <c r="A347" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="B347" t="s">
         <v>664</v>
@@ -7387,12 +7384,12 @@
         <v>100</v>
       </c>
       <c r="D347" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="348" spans="1:4">
       <c r="A348" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="B348" t="s">
         <v>665</v>
@@ -7401,12 +7398,12 @@
         <v>100</v>
       </c>
       <c r="D348" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="349" spans="1:4">
       <c r="A349" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="B349" t="s">
         <v>666</v>
@@ -7415,12 +7412,12 @@
         <v>100</v>
       </c>
       <c r="D349" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="350" spans="1:4">
       <c r="A350" t="s">
-        <v>291</v>
+        <v>219</v>
       </c>
       <c r="B350" t="s">
         <v>667</v>
@@ -7429,7 +7426,7 @@
         <v>100</v>
       </c>
       <c r="D350" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="351" spans="1:4">
@@ -7443,7 +7440,7 @@
         <v>100</v>
       </c>
       <c r="D351" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="352" spans="1:4">
@@ -7457,12 +7454,12 @@
         <v>100</v>
       </c>
       <c r="D352" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="353" spans="1:4">
       <c r="A353" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="B353" t="s">
         <v>670</v>
@@ -7471,7 +7468,7 @@
         <v>100</v>
       </c>
       <c r="D353" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="354" spans="1:4">
@@ -7485,7 +7482,7 @@
         <v>25</v>
       </c>
       <c r="D354" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="355" spans="1:4">
@@ -7499,7 +7496,7 @@
         <v>19</v>
       </c>
       <c r="D355" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="356" spans="1:4">
@@ -7513,7 +7510,7 @@
         <v>11200</v>
       </c>
       <c r="D356" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="357" spans="1:4">
@@ -7527,7 +7524,7 @@
         <v>3400</v>
       </c>
       <c r="D357" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="358" spans="1:4">
@@ -7541,7 +7538,7 @@
         <v>3200</v>
       </c>
       <c r="D358" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="359" spans="1:4">
@@ -7555,7 +7552,7 @@
         <v>1900</v>
       </c>
       <c r="D359" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="360" spans="1:4">
@@ -7569,7 +7566,7 @@
         <v>1100</v>
       </c>
       <c r="D360" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="361" spans="1:4">
@@ -7583,7 +7580,7 @@
         <v>1100</v>
       </c>
       <c r="D361" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="362" spans="1:4">
@@ -7597,7 +7594,7 @@
         <v>600</v>
       </c>
       <c r="D362" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="363" spans="1:4">
@@ -7611,7 +7608,7 @@
         <v>500</v>
       </c>
       <c r="D363" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="364" spans="1:4">
@@ -7625,12 +7622,12 @@
         <v>300</v>
       </c>
       <c r="D364" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="365" spans="1:4">
       <c r="A365" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="B365" t="s">
         <v>682</v>
@@ -7639,12 +7636,12 @@
         <v>200</v>
       </c>
       <c r="D365" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="366" spans="1:4">
       <c r="A366" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="B366" t="s">
         <v>683</v>
@@ -7653,7 +7650,7 @@
         <v>200</v>
       </c>
       <c r="D366" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="367" spans="1:4">
@@ -7667,12 +7664,12 @@
         <v>200</v>
       </c>
       <c r="D367" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="368" spans="1:4">
       <c r="A368" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="B368" t="s">
         <v>685</v>
@@ -7681,7 +7678,7 @@
         <v>100</v>
       </c>
       <c r="D368" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="369" spans="1:4">
@@ -7695,7 +7692,7 @@
         <v>100</v>
       </c>
       <c r="D369" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="370" spans="1:4">
@@ -7709,12 +7706,12 @@
         <v>100</v>
       </c>
       <c r="D370" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="371" spans="1:4">
       <c r="A371" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="B371" t="s">
         <v>688</v>
@@ -7723,7 +7720,7 @@
         <v>100</v>
       </c>
       <c r="D371" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="372" spans="1:4">
@@ -7737,7 +7734,7 @@
         <v>100</v>
       </c>
       <c r="D372" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="373" spans="1:4">
@@ -7751,7 +7748,7 @@
         <v>1000</v>
       </c>
       <c r="D373" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="374" spans="1:4">
@@ -7765,12 +7762,12 @@
         <v>900</v>
       </c>
       <c r="D374" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="375" spans="1:4">
       <c r="A375" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="B375" t="s">
         <v>692</v>
@@ -7779,7 +7776,7 @@
         <v>400</v>
       </c>
       <c r="D375" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="376" spans="1:4">
@@ -7793,7 +7790,7 @@
         <v>200</v>
       </c>
       <c r="D376" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="377" spans="1:4">
@@ -7807,7 +7804,7 @@
         <v>200</v>
       </c>
       <c r="D377" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="378" spans="1:4">
@@ -7821,7 +7818,7 @@
         <v>100</v>
       </c>
       <c r="D378" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="379" spans="1:4">
@@ -7835,7 +7832,7 @@
         <v>100</v>
       </c>
       <c r="D379" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="380" spans="1:4">
@@ -7849,7 +7846,7 @@
         <v>100</v>
       </c>
       <c r="D380" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="381" spans="1:4">
@@ -7863,7 +7860,7 @@
         <v>100</v>
       </c>
       <c r="D381" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="382" spans="1:4">
@@ -7877,7 +7874,7 @@
         <v>100</v>
       </c>
       <c r="D382" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="383" spans="1:4">
@@ -7891,12 +7888,12 @@
         <v>100</v>
       </c>
       <c r="D383" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="384" spans="1:4">
       <c r="A384" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="B384" t="s">
         <v>701</v>
@@ -7905,12 +7902,12 @@
         <v>100</v>
       </c>
       <c r="D384" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="385" spans="1:4">
       <c r="A385" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="B385" t="s">
         <v>702</v>
@@ -7919,7 +7916,7 @@
         <v>100</v>
       </c>
       <c r="D385" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="386" spans="1:4">
@@ -7933,7 +7930,7 @@
         <v>100</v>
       </c>
       <c r="D386" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="387" spans="1:4">
@@ -7947,12 +7944,12 @@
         <v>1000</v>
       </c>
       <c r="D387" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="388" spans="1:4">
       <c r="A388" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="B388" t="s">
         <v>705</v>
@@ -7961,7 +7958,7 @@
         <v>100</v>
       </c>
       <c r="D388" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="389" spans="1:4">
@@ -7975,7 +7972,7 @@
         <v>100</v>
       </c>
       <c r="D389" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="390" spans="1:4">
@@ -7989,7 +7986,7 @@
         <v>100</v>
       </c>
       <c r="D390" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="391" spans="1:4">
@@ -8003,12 +8000,12 @@
         <v>11708200</v>
       </c>
       <c r="D391" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="392" spans="1:4">
       <c r="A392" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="B392" t="s">
         <v>709</v>
@@ -8017,7 +8014,7 @@
         <v>1600</v>
       </c>
       <c r="D392" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="393" spans="1:4">
@@ -8031,12 +8028,12 @@
         <v>1000</v>
       </c>
       <c r="D393" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="394" spans="1:4">
       <c r="A394" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="B394" t="s">
         <v>711</v>
@@ -8045,7 +8042,7 @@
         <v>500</v>
       </c>
       <c r="D394" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="395" spans="1:4">
@@ -8059,7 +8056,7 @@
         <v>100</v>
       </c>
       <c r="D395" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="396" spans="1:4">
@@ -8073,7 +8070,7 @@
         <v>100</v>
       </c>
       <c r="D396" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="397" spans="1:4">
@@ -8087,7 +8084,7 @@
         <v>100</v>
       </c>
       <c r="D397" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="398" spans="1:4">
@@ -8101,7 +8098,7 @@
         <v>100</v>
       </c>
       <c r="D398" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="399" spans="1:4">
@@ -8115,21 +8112,7 @@
         <v>200</v>
       </c>
       <c r="D399" s="2">
-        <v>45786</v>
-      </c>
-    </row>
-    <row r="400" spans="1:4">
-      <c r="A400" t="s">
-        <v>270</v>
-      </c>
-      <c r="B400" t="s">
-        <v>717</v>
-      </c>
-      <c r="C400">
-        <v>500</v>
-      </c>
-      <c r="D400" s="2">
-        <v>45786</v>
+        <v>45788</v>
       </c>
     </row>
   </sheetData>

</xml_diff>